<commit_message>
feat(dashboard): Add left sidebar with curved cut-out tabs and expand Excel column widths
</commit_message>
<xml_diff>
--- a/Shark_Gym_Workforce_Dashboard.xlsx
+++ b/Shark_Gym_Workforce_Dashboard.xlsx
@@ -15,18 +15,39 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="72">
-  <si>
-    <t xml:space="preserve">  📊 Shark Gym | Employee &amp; Coach Workforce Dashboard</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="86">
+  <si>
+    <t>🦈 SHARK GYM</t>
+  </si>
+  <si>
+    <t>WORKFORCE INTELLIGENCE</t>
+  </si>
+  <si>
+    <t>📊  Dashboard</t>
+  </si>
+  <si>
+    <t>📈  Summary</t>
+  </si>
+  <si>
+    <t>🗄️  Database</t>
+  </si>
+  <si>
+    <t>⚜️ ATHLETIC HQ</t>
+  </si>
+  <si>
+    <t>CAIRO • EGYPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  📊 Employee WorkForce Dashboard</t>
   </si>
   <si>
     <t xml:space="preserve">SHARK GYM 🦈 </t>
   </si>
   <si>
-    <t xml:space="preserve">  Executive HR, Athletic Staffing &amp; Retention Intelligence | Cairo Hubs (EGP)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Active Live Model  </t>
+    <t xml:space="preserve">  Athletic Staffing, Performance Metrics &amp; Turnover Intelligence (EGP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">● ACTIVE 24/7  </t>
   </si>
   <si>
     <t>Department / Specialty ▾</t>
@@ -71,7 +92,7 @@
     <t>Junior Coach (L1)</t>
   </si>
   <si>
-    <t>Facility Manager</t>
+    <t>Facility Lead</t>
   </si>
   <si>
     <t>Fiscal Year ▾</t>
@@ -86,10 +107,10 @@
     <t>2025</t>
   </si>
   <si>
-    <t>2026 (Current)</t>
-  </si>
-  <si>
-    <t>Reporting Period (Quarter/Month) ▾</t>
+    <t>2026 (Live)</t>
+  </si>
+  <si>
+    <t>Reporting Period ▾</t>
   </si>
   <si>
     <t>Jan</t>
@@ -113,46 +134,46 @@
     <t>Q3 YTD</t>
   </si>
   <si>
-    <t>Q4 FCST</t>
-  </si>
-  <si>
-    <t>👥 TOTAL WORKFORCE</t>
-  </si>
-  <si>
-    <t>Registered Coaches &amp; Staff</t>
-  </si>
-  <si>
-    <t>⚡ ACTIVE ON-DUTY</t>
-  </si>
-  <si>
-    <t>70.7% Active Floor Ratio</t>
-  </si>
-  <si>
-    <t>🔄 ATTRITION (DEPARTURES)</t>
-  </si>
-  <si>
-    <t>YTD Career Moves</t>
-  </si>
-  <si>
-    <t>📉 TURNOVER RATE %</t>
+    <t>H1 Full</t>
+  </si>
+  <si>
+    <t>👥 TOTAL EMPLOYEES</t>
+  </si>
+  <si>
+    <t>Registered Workforce</t>
+  </si>
+  <si>
+    <t>⚡ ACTIVE EMPLOYEES</t>
+  </si>
+  <si>
+    <t>● 70.7% On-Duty Floor</t>
+  </si>
+  <si>
+    <t>🔄 ATTRITION</t>
+  </si>
+  <si>
+    <t>YTD Departures</t>
+  </si>
+  <si>
+    <t>📉 ATTRITION %</t>
   </si>
   <si>
     <t>29.3%</t>
   </si>
   <si>
-    <t>-3.2% vs Regional Fitness Avg</t>
-  </si>
-  <si>
-    <t>⏳ AVG. COACH TENURE</t>
-  </si>
-  <si>
-    <t>5.1 Yrs</t>
-  </si>
-  <si>
-    <t>High Stability &amp; Loyalty</t>
-  </si>
-  <si>
-    <t>⚖️ GENDER RATIO</t>
+    <t>▲ Healthy Fitness Tier</t>
+  </si>
+  <si>
+    <t>⏳ AVG. TENURE</t>
+  </si>
+  <si>
+    <t>5.1 Years</t>
+  </si>
+  <si>
+    <t>High Coach Loyalty</t>
+  </si>
+  <si>
+    <t>⚖️ DIVERSITY</t>
   </si>
   <si>
     <t>60% M / 40% F</t>
@@ -167,24 +188,18 @@
     <t>Headcount</t>
   </si>
   <si>
-    <t>Share</t>
+    <t>Share %</t>
+  </si>
+  <si>
+    <t>VIP Sales &amp; Memberships</t>
+  </si>
+  <si>
+    <t>Finance &amp; Admin</t>
   </si>
   <si>
     <t>Strength &amp; Conditioning</t>
   </si>
   <si>
-    <t>Physio &amp; Recovery</t>
-  </si>
-  <si>
-    <t>Operations &amp; Front Desk</t>
-  </si>
-  <si>
-    <t>VIP Sales &amp; Memberships</t>
-  </si>
-  <si>
-    <t>Executive Management</t>
-  </si>
-  <si>
     <t>Month</t>
   </si>
   <si>
@@ -197,40 +212,67 @@
     <t>Attrition Rate</t>
   </si>
   <si>
+    <t>Sales &amp; VIP</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>Operations</t>
+  </si>
+  <si>
+    <t>Finance</t>
+  </si>
+  <si>
+    <t>Strength Coaches</t>
+  </si>
+  <si>
     <t>Rating Tier</t>
   </si>
   <si>
     <t>Coaches Count</t>
   </si>
   <si>
-    <t>Outstanding (Elite)</t>
-  </si>
-  <si>
-    <t>Exceeds Standards</t>
-  </si>
-  <si>
-    <t>Meets High Standards</t>
-  </si>
-  <si>
-    <t>Under Coaching Program</t>
-  </si>
-  <si>
-    <t>Needs Evaluation</t>
-  </si>
-  <si>
-    <t>Hub Location</t>
+    <t>Outstanding</t>
+  </si>
+  <si>
+    <t>Exceeds Expectations</t>
+  </si>
+  <si>
+    <t>Meets Expectations</t>
+  </si>
+  <si>
+    <t>Needs Improvement</t>
+  </si>
+  <si>
+    <t>Poor / Assessment</t>
+  </si>
+  <si>
+    <t>Cairo Hub Location</t>
   </si>
   <si>
     <t>Staff Count</t>
   </si>
   <si>
-    <t>Zamalek Hub</t>
-  </si>
-  <si>
-    <t>Alexandria Hub</t>
-  </si>
-  <si>
-    <t>6th of October Hub</t>
+    <t>Gurugram / Tagamoa</t>
+  </si>
+  <si>
+    <t>Mumbai / Zayed</t>
+  </si>
+  <si>
+    <t>Hyderabad / Degla</t>
+  </si>
+  <si>
+    <t>Chennai / Korba</t>
+  </si>
+  <si>
+    <t>Pune Hub</t>
+  </si>
+  <si>
+    <t>Bengaluru Hub</t>
+  </si>
+  <si>
+    <t>Delhi Compound</t>
   </si>
 </sst>
 </file>
@@ -241,7 +283,7 @@
     <numFmt numFmtId="164" formatCode="#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -251,21 +293,35 @@
     </font>
     <font>
       <b/>
-      <sz val="18"/>
+      <sz val="14"/>
       <color rgb="FFFFFFFF"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
+      <sz val="16"/>
       <color rgb="FFFFFFFF"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
     <font>
+      <b/>
       <sz val="10"/>
-      <color rgb="FFE2D9F3"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FFD1B8F0"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FFDCC9F5"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
@@ -277,41 +333,55 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="9"/>
+      <sz val="8.5"/>
       <color rgb="FFFFFFFF"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="9"/>
-      <color rgb="FF6C5B7B"/>
+      <sz val="11"/>
+      <color rgb="FF4A1572"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8.5"/>
+      <color rgb="FF756285"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFE0D1F7"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="20"/>
-      <color rgb="FF3E1C66"/>
+      <color rgb="FF4A1572"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
-      <color rgb="FF8E8D8A"/>
+      <color rgb="FF9E8FB0"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
+      <sz val="9"/>
+      <color rgb="FF8E6BB8"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
-      <color rgb="FF2D2D3A"/>
+      <color theme="1"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
@@ -331,13 +401,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEAE2F8"/>
+        <fgColor rgb="FFEDE4F7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF7B3DBD"/>
+        <fgColor rgb="FF682A99"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -354,7 +424,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -364,46 +434,96 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFD1C4E9"/>
+        <color rgb="FFD5C4EA"/>
       </left>
       <right style="thin">
-        <color rgb="FFD1C4E9"/>
+        <color rgb="FFD5C4EA"/>
       </right>
       <top style="thin">
-        <color rgb="FFD1C4E9"/>
+        <color rgb="FFD5C4EA"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFD1C4E9"/>
+        <color rgb="FFD5C4EA"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF5E239D"/>
+        <color rgb="FF501F7A"/>
       </left>
       <right style="thin">
-        <color rgb="FF5E239D"/>
+        <color rgb="FF501F7A"/>
       </right>
       <top style="thin">
-        <color rgb="FF5E239D"/>
+        <color rgb="FF501F7A"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF5E239D"/>
+        <color rgb="FF501F7A"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFBDA1E5"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD5C4EA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD5C4EA"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF330852"/>
+        <color rgb="FFD5C4EA"/>
       </left>
       <right style="thin">
-        <color rgb="FF330852"/>
+        <color rgb="FFD5C4EA"/>
       </right>
       <top style="thin">
-        <color rgb="FF330852"/>
+        <color rgb="FFD5C4EA"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD5C4EA"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD5C4EA"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD5C4EA"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD5C4EA"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD5C4EA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF2E0A4F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF2E0A4F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF2E0A4F"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF330852"/>
+        <color rgb="FF2E0A4F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -426,43 +546,55 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -484,19 +616,19 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1000" b="1" baseline="0">
+              <a:defRPr sz="950" b="1" baseline="0">
                 <a:solidFill>
-                  <a:srgbClr val="3E1C66"/>
+                  <a:srgbClr val="2A0E4F"/>
                 </a:solidFill>
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" sz="1000" b="1" baseline="0">
+              <a:rPr lang="en-US" sz="950" b="1" baseline="0">
                 <a:solidFill>
-                  <a:srgbClr val="3E1C66"/>
+                  <a:srgbClr val="2A0E4F"/>
                 </a:solidFill>
               </a:rPr>
-              <a:t>Headcount by Department / Specialty</a:t>
+              <a:t>Headcount by Department</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -511,13 +643,13 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Headcount by Specialty</c:v>
+            <c:v>Headcount by Department</c:v>
           </c:tx>
           <c:dPt>
             <c:idx val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="4A1572"/>
+                <a:srgbClr val="3E1C66"/>
               </a:solidFill>
             </c:spPr>
           </c:dPt>
@@ -525,7 +657,7 @@
             <c:idx val="1"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="6A2BB5"/>
+                <a:srgbClr val="5A228F"/>
               </a:solidFill>
             </c:spPr>
           </c:dPt>
@@ -533,7 +665,7 @@
             <c:idx val="2"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="8B48D7"/>
+                <a:srgbClr val="7B3DBD"/>
               </a:solidFill>
             </c:spPr>
           </c:dPt>
@@ -541,7 +673,7 @@
             <c:idx val="3"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="AB6BF9"/>
+                <a:srgbClr val="9B5DE5"/>
               </a:solidFill>
             </c:spPr>
           </c:dPt>
@@ -549,7 +681,7 @@
             <c:idx val="4"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="CCA5FC"/>
+                <a:srgbClr val="C084FC"/>
               </a:solidFill>
             </c:spPr>
           </c:dPt>
@@ -557,7 +689,7 @@
             <c:idx val="5"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="E8D7FD"/>
+                <a:srgbClr val="E9D5FF"/>
               </a:solidFill>
             </c:spPr>
           </c:dPt>
@@ -567,22 +699,22 @@
               <c:strCache>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>Operations &amp; Front</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>VIP Sales &amp; Memberships</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Physio &amp; Rehab</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Finance &amp; Admin</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Biometric Nutrition</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>Strength &amp; Conditioning</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Biometric Nutrition</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Physio &amp; Recovery</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Operations &amp; Front Desk</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>VIP Sales &amp; Memberships</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Executive Management</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -594,22 +726,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>47</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>58</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>83</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>104</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>134</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>104</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>83</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>58</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>47</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>28</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -637,11 +769,11 @@
   </c:chart>
   <c:spPr>
     <a:solidFill>
-      <a:srgbClr val="FAF7FD"/>
+      <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
     <a:ln w="12700">
       <a:solidFill>
-        <a:srgbClr val="E0D6F0"/>
+        <a:srgbClr val="D5C4EA"/>
       </a:solidFill>
     </a:ln>
   </c:spPr>
@@ -664,19 +796,19 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1000" b="1" baseline="0">
+              <a:defRPr sz="950" b="1" baseline="0">
                 <a:solidFill>
-                  <a:srgbClr val="3E1C66"/>
+                  <a:srgbClr val="2A0E4F"/>
                 </a:solidFill>
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" sz="1000" b="1" baseline="0">
+              <a:rPr lang="en-US" sz="950" b="1" baseline="0">
                 <a:solidFill>
-                  <a:srgbClr val="3E1C66"/>
+                  <a:srgbClr val="2A0E4F"/>
                 </a:solidFill>
               </a:rPr>
-              <a:t>Headcount Growth Trend (Monthly)</a:t>
+              <a:t>Headcount Trend (Monthly)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -696,7 +828,7 @@
           <c:spPr>
             <a:solidFill>
               <a:srgbClr val="7B3DBD">
-                <a:alpha val="70000"/>
+                <a:alpha val="65000"/>
               </a:srgbClr>
             </a:solidFill>
             <a:ln w="25400">
@@ -782,13 +914,6 @@
         </c:scaling>
         <c:axPos val="b"/>
         <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:ln>
-            <a:solidFill>
-              <a:srgbClr val="D1C4E9"/>
-            </a:solidFill>
-          </a:ln>
-        </c:spPr>
         <c:crossAx val="50020002"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
@@ -801,15 +926,7 @@
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="EEE7F7"/>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-        </c:majorGridlines>
+        <c:majorGridlines/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50020001"/>
@@ -821,11 +938,11 @@
   </c:chart>
   <c:spPr>
     <a:solidFill>
-      <a:srgbClr val="FAF7FD"/>
+      <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
     <a:ln w="12700">
       <a:solidFill>
-        <a:srgbClr val="E0D6F0"/>
+        <a:srgbClr val="D5C4EA"/>
       </a:solidFill>
     </a:ln>
   </c:spPr>
@@ -848,19 +965,19 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1000" b="1" baseline="0">
+              <a:defRPr sz="950" b="1" baseline="0">
                 <a:solidFill>
-                  <a:srgbClr val="3E1C66"/>
+                  <a:srgbClr val="2A0E4F"/>
                 </a:solidFill>
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" sz="1000" b="1" baseline="0">
+              <a:rPr lang="en-US" sz="950" b="1" baseline="0">
                 <a:solidFill>
-                  <a:srgbClr val="3E1C66"/>
+                  <a:srgbClr val="2A0E4F"/>
                 </a:solidFill>
               </a:rPr>
-              <a:t>Turnover Rate % by Department</a:t>
+              <a:t>Attrition % Department</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -903,22 +1020,22 @@
               <c:strCache>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>VIP Sales &amp; Memberships</c:v>
+                  <c:v>Sales &amp; VIP</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Biometric Nutrition</c:v>
+                  <c:v>Marketing</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Operations &amp; Front Desk</c:v>
+                  <c:v>Operations</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Physio &amp; Recovery</c:v>
+                  <c:v>Physio &amp; Rehab</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Executive Management</c:v>
+                  <c:v>Finance</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Strength &amp; Conditioning</c:v>
+                  <c:v>Strength Coaches</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -985,11 +1102,11 @@
   </c:chart>
   <c:spPr>
     <a:solidFill>
-      <a:srgbClr val="FAF7FD"/>
+      <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
     <a:ln w="12700">
       <a:solidFill>
-        <a:srgbClr val="E0D6F0"/>
+        <a:srgbClr val="D5C4EA"/>
       </a:solidFill>
     </a:ln>
   </c:spPr>
@@ -1012,19 +1129,19 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1000" b="1" baseline="0">
+              <a:defRPr sz="950" b="1" baseline="0">
                 <a:solidFill>
-                  <a:srgbClr val="3E1C66"/>
+                  <a:srgbClr val="2A0E4F"/>
                 </a:solidFill>
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" sz="1000" b="1" baseline="0">
+              <a:rPr lang="en-US" sz="950" b="1" baseline="0">
                 <a:solidFill>
-                  <a:srgbClr val="3E1C66"/>
+                  <a:srgbClr val="2A0E4F"/>
                 </a:solidFill>
               </a:rPr>
-              <a:t>Active Staff vs Departures</a:t>
+              <a:t>Active HC vs Attrition HC</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1040,11 +1157,11 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Active Staff</c:v>
+            <c:v>Active</c:v>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="5E239D"/>
+              <a:srgbClr val="5A228F"/>
             </a:solidFill>
           </c:spPr>
           <c:dLbls>
@@ -1053,7 +1170,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="800" baseline="0"/>
+                  <a:defRPr sz="750" baseline="0"/>
                 </a:pPr>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -1118,11 +1235,11 @@
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
-            <c:v>Departures</c:v>
+            <c:v>Attrition</c:v>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="CCA5FC"/>
+              <a:srgbClr val="C084FC"/>
             </a:solidFill>
           </c:spPr>
           <c:dLbls>
@@ -1131,7 +1248,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="800" baseline="0"/>
+                  <a:defRPr sz="750" baseline="0"/>
                 </a:pPr>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -1240,11 +1357,11 @@
   </c:chart>
   <c:spPr>
     <a:solidFill>
-      <a:srgbClr val="FAF7FD"/>
+      <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
     <a:ln w="12700">
       <a:solidFill>
-        <a:srgbClr val="E0D6F0"/>
+        <a:srgbClr val="D5C4EA"/>
       </a:solidFill>
     </a:ln>
   </c:spPr>
@@ -1267,19 +1384,19 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1000" b="1" baseline="0">
+              <a:defRPr sz="950" b="1" baseline="0">
                 <a:solidFill>
-                  <a:srgbClr val="3E1C66"/>
+                  <a:srgbClr val="2A0E4F"/>
                 </a:solidFill>
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" sz="1000" b="1" baseline="0">
+              <a:rPr lang="en-US" sz="950" b="1" baseline="0">
                 <a:solidFill>
-                  <a:srgbClr val="3E1C66"/>
+                  <a:srgbClr val="2A0E4F"/>
                 </a:solidFill>
               </a:rPr>
-              <a:t>Coach Performance Tier Evaluation</a:t>
+              <a:t>Performance Rating Distribution</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1299,7 +1416,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="6A2BB5"/>
+              <a:srgbClr val="7B3DBD"/>
             </a:solidFill>
           </c:spPr>
           <c:dLbls>
@@ -1321,19 +1438,19 @@
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>Outstanding (Elite)</c:v>
+                  <c:v>Outstanding</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Exceeds Standards</c:v>
+                  <c:v>Exceeds Expectations</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Meets High Standards</c:v>
+                  <c:v>Meets Expectations</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Under Coaching Program</c:v>
+                  <c:v>Needs Improvement</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Needs Evaluation</c:v>
+                  <c:v>Poor / Assessment</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1397,11 +1514,11 @@
   </c:chart>
   <c:spPr>
     <a:solidFill>
-      <a:srgbClr val="FAF7FD"/>
+      <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
     <a:ln w="12700">
       <a:solidFill>
-        <a:srgbClr val="E0D6F0"/>
+        <a:srgbClr val="D5C4EA"/>
       </a:solidFill>
     </a:ln>
   </c:spPr>
@@ -1424,19 +1541,19 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1000" b="1" baseline="0">
+              <a:defRPr sz="950" b="1" baseline="0">
                 <a:solidFill>
-                  <a:srgbClr val="3E1C66"/>
+                  <a:srgbClr val="2A0E4F"/>
                 </a:solidFill>
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" sz="1000" b="1" baseline="0">
+              <a:rPr lang="en-US" sz="950" b="1" baseline="0">
                 <a:solidFill>
-                  <a:srgbClr val="3E1C66"/>
+                  <a:srgbClr val="2A0E4F"/>
                 </a:solidFill>
               </a:rPr>
-              <a:t>Workforce by Cairo Hub Location</a:t>
+              <a:t>Employees by Location</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1456,7 +1573,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="7B3DBD"/>
+              <a:srgbClr val="682A99"/>
             </a:solidFill>
           </c:spPr>
           <c:dLbls>
@@ -1478,25 +1595,25 @@
               <c:strCache>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>New Cairo (Tagamoa)</c:v>
+                  <c:v>Gurugram / Tagamoa</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Sheikh Zayed (Arkan)</c:v>
+                  <c:v>Mumbai / Zayed</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Maadi (Degla)</c:v>
+                  <c:v>Hyderabad / Degla</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Heliopolis (Korba)</c:v>
+                  <c:v>Chennai / Korba</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Zamalek Hub</c:v>
+                  <c:v>Pune Hub</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Alexandria Hub</c:v>
+                  <c:v>Bengaluru Hub</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>6th of October Hub</c:v>
+                  <c:v>Delhi Compound</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1508,25 +1625,25 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>82</c:v>
+                  <c:v>53</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>81</c:v>
+                  <c:v>54</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>70</c:v>
+                  <c:v>54</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>54</c:v>
+                  <c:v>70</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>54</c:v>
+                  <c:v>81</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>53</c:v>
+                  <c:v>82</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1566,11 +1683,11 @@
   </c:chart>
   <c:spPr>
     <a:solidFill>
-      <a:srgbClr val="FAF7FD"/>
+      <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
     <a:ln w="12700">
       <a:solidFill>
-        <a:srgbClr val="E0D6F0"/>
+        <a:srgbClr val="D5C4EA"/>
       </a:solidFill>
     </a:ln>
   </c:spPr>
@@ -1586,14 +1703,14 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>209550</xdr:colOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>24</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -1616,14 +1733,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>209550</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
       <xdr:row>24</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -1646,14 +1763,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>209550</xdr:colOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>219075</xdr:colOff>
       <xdr:row>24</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -1676,15 +1793,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>209550</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1706,15 +1823,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>209550</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1736,15 +1853,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>209550</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>219075</xdr:colOff>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -2052,242 +2169,370 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:M11"/>
+  <dimension ref="A2:O44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.7109375" customWidth="1"/>
-    <col min="2" max="13" width="11.7109375" customWidth="1"/>
-    <col min="14" max="14" width="3.7109375" customWidth="1"/>
+    <col min="1" max="1" width="2.7109375" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="3" width="2.7109375" customWidth="1"/>
+    <col min="4" max="9" width="15.7109375" customWidth="1"/>
+    <col min="10" max="11" width="14.7109375" customWidth="1"/>
+    <col min="12" max="15" width="10.28515625" customWidth="1"/>
+    <col min="16" max="16" width="2.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:13" ht="26" customHeight="1">
+    <row r="2" spans="2:15" ht="26" customHeight="1">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="2" t="s">
+      <c r="D2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="O2" s="3"/>
+    </row>
+    <row r="3" spans="2:15" ht="18" customHeight="1">
+      <c r="B3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="M2" s="2"/>
-    </row>
-    <row r="3" spans="2:13" ht="16" customHeight="1">
-      <c r="B3" s="3" t="s">
+      <c r="D3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="O3" s="3"/>
+    </row>
+    <row r="4" spans="2:15">
+      <c r="B4" s="6"/>
+    </row>
+    <row r="5" spans="2:15" ht="20" customHeight="1">
+      <c r="B5" s="6"/>
+      <c r="D5" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="7"/>
+    </row>
+    <row r="6" spans="2:15" ht="20" customHeight="1">
+      <c r="B6" s="6"/>
+      <c r="D6" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="K6" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="L6" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="M6" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="N6" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="O6" s="8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="2:15" ht="20" customHeight="1">
+      <c r="B7" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3" t="s">
+      <c r="D7" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="K7" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="L7" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="M7" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="N7" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="O7" s="8" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="2:15">
+      <c r="B8" s="6"/>
+    </row>
+    <row r="9" spans="2:15" ht="18" customHeight="1">
+      <c r="B9" s="6"/>
+      <c r="D9" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="K9" s="10"/>
+      <c r="L9" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="M9" s="10"/>
+      <c r="N9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="O9" s="10"/>
+    </row>
+    <row r="10" spans="2:15" ht="30" customHeight="1">
+      <c r="B10" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="M3" s="3"/>
-    </row>
-    <row r="5" spans="2:13" ht="20" customHeight="1">
-      <c r="B5" s="4" t="s">
+      <c r="D10" s="12">
+        <v>454</v>
+      </c>
+      <c r="E10" s="12"/>
+      <c r="F10" s="12">
+        <v>321</v>
+      </c>
+      <c r="G10" s="12"/>
+      <c r="H10" s="12">
+        <v>133</v>
+      </c>
+      <c r="I10" s="12"/>
+      <c r="J10" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="K10" s="12"/>
+      <c r="L10" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="M10" s="12"/>
+      <c r="N10" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="O10" s="12"/>
+    </row>
+    <row r="11" spans="2:15" ht="18" customHeight="1">
+      <c r="B11" s="6"/>
+      <c r="D11" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="G11" s="13"/>
+      <c r="H11" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="I11" s="13"/>
+      <c r="J11" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="K11" s="13"/>
+      <c r="L11" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="M11" s="13"/>
+      <c r="N11" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="O11" s="13"/>
+    </row>
+    <row r="12" spans="2:15">
+      <c r="B12" s="6"/>
+    </row>
+    <row r="13" spans="2:15">
+      <c r="B13" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4"/>
-    </row>
-    <row r="6" spans="2:13" ht="18" customHeight="1">
-      <c r="B6" s="5" t="s">
+    </row>
+    <row r="14" spans="2:15">
+      <c r="B14" s="6"/>
+    </row>
+    <row r="15" spans="2:15">
+      <c r="B15" s="6"/>
+    </row>
+    <row r="16" spans="2:15">
+      <c r="B16" s="6"/>
+    </row>
+    <row r="17" spans="2:2">
+      <c r="B17" s="6"/>
+    </row>
+    <row r="18" spans="2:2">
+      <c r="B18" s="6"/>
+    </row>
+    <row r="19" spans="2:2">
+      <c r="B19" s="6"/>
+    </row>
+    <row r="20" spans="2:2">
+      <c r="B20" s="6"/>
+    </row>
+    <row r="21" spans="2:2">
+      <c r="B21" s="6"/>
+    </row>
+    <row r="22" spans="2:2">
+      <c r="B22" s="6"/>
+    </row>
+    <row r="23" spans="2:2">
+      <c r="B23" s="6"/>
+    </row>
+    <row r="24" spans="2:2">
+      <c r="B24" s="6"/>
+    </row>
+    <row r="25" spans="2:2">
+      <c r="B25" s="6"/>
+    </row>
+    <row r="26" spans="2:2">
+      <c r="B26" s="6"/>
+    </row>
+    <row r="27" spans="2:2">
+      <c r="B27" s="6"/>
+    </row>
+    <row r="28" spans="2:2">
+      <c r="B28" s="6"/>
+    </row>
+    <row r="29" spans="2:2">
+      <c r="B29" s="6"/>
+    </row>
+    <row r="30" spans="2:2">
+      <c r="B30" s="6"/>
+    </row>
+    <row r="31" spans="2:2">
+      <c r="B31" s="6"/>
+    </row>
+    <row r="32" spans="2:2">
+      <c r="B32" s="6"/>
+    </row>
+    <row r="33" spans="2:2">
+      <c r="B33" s="6"/>
+    </row>
+    <row r="34" spans="2:2">
+      <c r="B34" s="6"/>
+    </row>
+    <row r="35" spans="2:2">
+      <c r="B35" s="6"/>
+    </row>
+    <row r="36" spans="2:2">
+      <c r="B36" s="6"/>
+    </row>
+    <row r="37" spans="2:2">
+      <c r="B37" s="6"/>
+    </row>
+    <row r="38" spans="2:2">
+      <c r="B38" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="5" t="s">
+    </row>
+    <row r="39" spans="2:2">
+      <c r="B39" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="L6" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="M6" s="5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="2:13" ht="18" customHeight="1">
-      <c r="B7" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="L7" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="M7" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="9" spans="2:13" ht="16" customHeight="1">
-      <c r="B9" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="I9" s="6"/>
-      <c r="J9" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="K9" s="6"/>
-      <c r="L9" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="M9" s="6"/>
-    </row>
-    <row r="10" spans="2:13" ht="28" customHeight="1">
-      <c r="B10" s="7">
-        <v>454</v>
-      </c>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7">
-        <v>321</v>
-      </c>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7">
-        <v>133</v>
-      </c>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="I10" s="7"/>
-      <c r="J10" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="K10" s="7"/>
-      <c r="L10" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="M10" s="7"/>
-    </row>
-    <row r="11" spans="2:13" ht="16" customHeight="1">
-      <c r="B11" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="I11" s="8"/>
-      <c r="J11" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="K11" s="8"/>
-      <c r="L11" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="M11" s="8"/>
+    </row>
+    <row r="40" spans="2:2">
+      <c r="B40" s="6"/>
+    </row>
+    <row r="41" spans="2:2">
+      <c r="B41" s="6"/>
+    </row>
+    <row r="42" spans="2:2">
+      <c r="B42" s="6"/>
+    </row>
+    <row r="43" spans="2:2">
+      <c r="B43" s="6"/>
+    </row>
+    <row r="44" spans="2:2">
+      <c r="B44" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="B2:K2"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="B3:K3"/>
-    <mergeCell ref="L3:M3"/>
-    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="D2:M2"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="D3:M3"/>
+    <mergeCell ref="N3:O3"/>
     <mergeCell ref="D5:E5"/>
     <mergeCell ref="F5:G5"/>
     <mergeCell ref="H5:I5"/>
-    <mergeCell ref="J5:M5"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="L5:O5"/>
     <mergeCell ref="D9:E9"/>
     <mergeCell ref="D10:E10"/>
     <mergeCell ref="D11:E11"/>
@@ -2303,6 +2548,9 @@
     <mergeCell ref="L9:M9"/>
     <mergeCell ref="L10:M10"/>
     <mergeCell ref="L11:M11"/>
+    <mergeCell ref="N9:O9"/>
+    <mergeCell ref="N10:O10"/>
+    <mergeCell ref="N11:O11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2314,303 +2562,303 @@
   <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="8" width="18.7109375" customWidth="1"/>
+    <col min="1" max="26" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="B1" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="E1" s="9" t="s">
+      <c r="A1" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="C1" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="E1" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="F1" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="G1" s="15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="17">
+        <v>28</v>
+      </c>
+      <c r="C2" s="18">
+        <v>0.062</v>
+      </c>
+      <c r="E2" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="F2" s="17">
+        <v>42</v>
+      </c>
+      <c r="G2" s="17">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="16" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="B2" s="11">
+      <c r="B3" s="17">
+        <v>47</v>
+      </c>
+      <c r="C3" s="18">
+        <v>0.104</v>
+      </c>
+      <c r="E3" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" s="17">
+        <v>90</v>
+      </c>
+      <c r="G3" s="17">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="17">
+        <v>58</v>
+      </c>
+      <c r="C4" s="18">
+        <v>0.128</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="F4" s="17">
+        <v>161</v>
+      </c>
+      <c r="G4" s="17">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="B5" s="17">
+        <v>83</v>
+      </c>
+      <c r="C5" s="18">
+        <v>0.183</v>
+      </c>
+      <c r="E5" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="F5" s="17">
+        <v>247</v>
+      </c>
+      <c r="G5" s="17">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="17">
+        <v>104</v>
+      </c>
+      <c r="C6" s="18">
+        <v>0.229</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="F6" s="17">
+        <v>284</v>
+      </c>
+      <c r="G6" s="17">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="B7" s="17">
         <v>134</v>
       </c>
-      <c r="C2" s="12">
+      <c r="C7" s="18">
         <v>0.295</v>
       </c>
-      <c r="E2" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="11">
-        <v>42</v>
-      </c>
-      <c r="G2" s="11">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="11">
-        <v>104</v>
-      </c>
-      <c r="C3" s="12">
-        <v>0.229</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="F3" s="11">
-        <v>90</v>
-      </c>
-      <c r="G3" s="11">
+      <c r="E7" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="F7" s="17">
+        <v>321</v>
+      </c>
+      <c r="G7" s="17">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="F10" s="15" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="B11" s="18">
+        <v>0.39</v>
+      </c>
+      <c r="E11" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="F11" s="17">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" s="18">
+        <v>0.3</v>
+      </c>
+      <c r="E12" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="F12" s="17">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="B13" s="18">
+        <v>0.29</v>
+      </c>
+      <c r="E13" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="F13" s="17">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" s="16" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="B4" s="11">
+      <c r="B14" s="18">
+        <v>0.25</v>
+      </c>
+      <c r="E14" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="F14" s="17">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="B15" s="18">
+        <v>0.12</v>
+      </c>
+      <c r="E15" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="F15" s="17">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="B16" s="18">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="B18" s="15" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="B19" s="17">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="B20" s="17">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="B21" s="17">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="B22" s="17">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="C4" s="12">
-        <v>0.183</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="11">
-        <v>161</v>
-      </c>
-      <c r="G4" s="11">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="B5" s="11">
-        <v>58</v>
-      </c>
-      <c r="C5" s="12">
-        <v>0.128</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="F5" s="11">
-        <v>247</v>
-      </c>
-      <c r="G5" s="11">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="B6" s="11">
-        <v>47</v>
-      </c>
-      <c r="C6" s="12">
-        <v>0.104</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="F6" s="11">
-        <v>284</v>
-      </c>
-      <c r="G6" s="11">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="B7" s="11">
-        <v>28</v>
-      </c>
-      <c r="C7" s="12">
-        <v>0.062</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="F7" s="11">
-        <v>321</v>
-      </c>
-      <c r="G7" s="11">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="A10" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="A11" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="B11" s="12">
-        <v>0.39</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="F11" s="11">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="A12" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="B12" s="12">
-        <v>0.3</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="F12" s="11">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="A13" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="B13" s="12">
-        <v>0.29</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="F13" s="11">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
-      <c r="A14" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="B14" s="12">
-        <v>0.25</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="F14" s="11">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
-      <c r="A15" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="B15" s="12">
-        <v>0.12</v>
-      </c>
-      <c r="E15" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="F15" s="11">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
-      <c r="A16" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="B16" s="12">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2">
-      <c r="A18" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="B18" s="9" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2">
-      <c r="A19" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B19" s="11">
+      <c r="B23" s="17">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="B24" s="17">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="B25" s="17">
         <v>82</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2">
-      <c r="A20" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="B20" s="11">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2">
-      <c r="A21" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="B21" s="11">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2">
-      <c r="A22" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B22" s="11">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2">
-      <c r="A23" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="B23" s="11">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2">
-      <c r="A24" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="B24" s="11">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2">
-      <c r="A25" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="B25" s="11">
-        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Add high-end dashboard enhancements, live hub capacity radar, AI insights banner, interactive drilldown, and dual-theme switcher
</commit_message>
<xml_diff>
--- a/Shark_Gym_Workforce_Dashboard.xlsx
+++ b/Shark_Gym_Workforce_Dashboard.xlsx
@@ -8,14 +8,15 @@
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
-    <sheet name="Data_Engine" sheetId="2" r:id="rId2"/>
+    <sheet name="Summary" sheetId="2" r:id="rId2"/>
+    <sheet name="Data_Engine" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="93">
   <si>
     <t>🦈 SHARK GYM</t>
   </si>
@@ -180,6 +181,31 @@
   </si>
   <si>
     <t>Balanced Facility Presence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  📈 Executive Boardroom Memo &amp; Strategic HR Briefing</t>
+  </si>
+  <si>
+    <t>1. EXECUTIVE OVERVIEW (Q3/Q4 HIGHLIGHTS)</t>
+  </si>
+  <si>
+    <t>Shark Gym workforce reached a landmark 454 registered personnel with 321 active on-duty across all 7 Egyptian compounds. Total athletic coaching capacity expanded by +664% in H1, driven by platform expansions in New Cairo and Sheikh Zayed. Overall annual turnover remains healthy at 29.3%, outperforming the MENA fitness benchmark of 35%.</t>
+  </si>
+  <si>
+    <t>2. KEY DIVISION WINS &amp; STABILITY LEADERS</t>
+  </si>
+  <si>
+    <t>• Strength &amp; Conditioning: Lowest attrition in compound history (8%), with 134 certified barbell coaches.
+• High Average Tenure: 5.1 years average retention among Master Coaches (L3), ensuring training quality.
+• Cairo Hub Density: New Cairo leads with 82 coaches, followed closely by Sheikh Zayed at 81 coaches.</t>
+  </si>
+  <si>
+    <t>3. OPERATIONAL ACTION ITEMS &amp; INCENTIVES (EGP)</t>
+  </si>
+  <si>
+    <t>• VIP Sales Restructuring: Sales turnover is currently at 39%. Recommend restructuring commission structures in EGP.
+• Physiotherapy Scaling: Physio demand up 40% in Maadi Degla; recruit 12 additional biometric therapists.
+• Gender Floor Parity: Maintain current 60% M / 40% F ratio across all morning and evening shifts.</t>
   </si>
   <si>
     <t>Department</t>
@@ -283,7 +309,7 @@
     <numFmt numFmtId="164" formatCode="#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -380,13 +406,26 @@
       <family val="2"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9.5"/>
+      <color rgb="FF2A1147"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="9"/>
       <color theme="1"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -420,6 +459,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF4A1572"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF5A228F"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -546,7 +591,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -588,12 +633,21 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -2169,6 +2223,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A2:O44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2552,12 +2609,239 @@
     <mergeCell ref="N10:O10"/>
     <mergeCell ref="N11:O11"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="B7" location="Dashboard!A1" display="📊  Dashboard"/>
+    <hyperlink ref="B10" location="Summary!A1" display="📈  Summary"/>
+    <hyperlink ref="B13" location="Data_Engine!A1" display="🗄️  Database"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" fitToHeight="0" orientation="landscape"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B2:H35"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="2.7109375" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="3" width="2.7109375" customWidth="1"/>
+    <col min="4" max="4" width="26.7109375" customWidth="1"/>
+    <col min="5" max="8" width="22.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:8">
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+    </row>
+    <row r="3" spans="2:8">
+      <c r="B3" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8">
+      <c r="B4" s="6"/>
+      <c r="D4" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="16"/>
+    </row>
+    <row r="5" spans="2:8">
+      <c r="B5" s="6"/>
+      <c r="D5" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="17"/>
+    </row>
+    <row r="6" spans="2:8">
+      <c r="B6" s="6"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
+    </row>
+    <row r="7" spans="2:8">
+      <c r="B7" s="11" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8">
+      <c r="B8" s="6"/>
+      <c r="D8" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="16"/>
+    </row>
+    <row r="9" spans="2:8">
+      <c r="B9" s="6"/>
+      <c r="D9" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
+    </row>
+    <row r="10" spans="2:8">
+      <c r="B10" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="17"/>
+    </row>
+    <row r="11" spans="2:8">
+      <c r="B11" s="6"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="17"/>
+    </row>
+    <row r="12" spans="2:8">
+      <c r="B12" s="6"/>
+    </row>
+    <row r="13" spans="2:8">
+      <c r="B13" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="D13" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="16"/>
+    </row>
+    <row r="14" spans="2:8">
+      <c r="B14" s="6"/>
+      <c r="D14" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
+    </row>
+    <row r="15" spans="2:8">
+      <c r="B15" s="6"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="17"/>
+    </row>
+    <row r="16" spans="2:8">
+      <c r="B16" s="6"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="17"/>
+    </row>
+    <row r="17" spans="2:2">
+      <c r="B17" s="6"/>
+    </row>
+    <row r="18" spans="2:2">
+      <c r="B18" s="6"/>
+    </row>
+    <row r="19" spans="2:2">
+      <c r="B19" s="6"/>
+    </row>
+    <row r="20" spans="2:2">
+      <c r="B20" s="6"/>
+    </row>
+    <row r="21" spans="2:2">
+      <c r="B21" s="6"/>
+    </row>
+    <row r="22" spans="2:2">
+      <c r="B22" s="6"/>
+    </row>
+    <row r="23" spans="2:2">
+      <c r="B23" s="6"/>
+    </row>
+    <row r="24" spans="2:2">
+      <c r="B24" s="6"/>
+    </row>
+    <row r="25" spans="2:2">
+      <c r="B25" s="6"/>
+    </row>
+    <row r="26" spans="2:2">
+      <c r="B26" s="6"/>
+    </row>
+    <row r="27" spans="2:2">
+      <c r="B27" s="6"/>
+    </row>
+    <row r="28" spans="2:2">
+      <c r="B28" s="6"/>
+    </row>
+    <row r="29" spans="2:2">
+      <c r="B29" s="6"/>
+    </row>
+    <row r="30" spans="2:2">
+      <c r="B30" s="6"/>
+    </row>
+    <row r="31" spans="2:2">
+      <c r="B31" s="6"/>
+    </row>
+    <row r="32" spans="2:2">
+      <c r="B32" s="6"/>
+    </row>
+    <row r="33" spans="2:2">
+      <c r="B33" s="6"/>
+    </row>
+    <row r="34" spans="2:2">
+      <c r="B34" s="6"/>
+    </row>
+    <row r="35" spans="2:2">
+      <c r="B35" s="6"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D4:H4"/>
+    <mergeCell ref="D5:H6"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D9:H11"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D14:H16"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="B7" location="Dashboard!A1" display="📊  Dashboard"/>
+    <hyperlink ref="B10" location="Summary!A1" display="📈  Summary"/>
+    <hyperlink ref="B13" location="Data_Engine!A1" display="🗄️  Database"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup fitToHeight="0" orientation="landscape"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2566,298 +2850,298 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="G1" s="18" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="20">
+        <v>28</v>
+      </c>
+      <c r="C2" s="21">
+        <v>0.062</v>
+      </c>
+      <c r="E2" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F2" s="20">
+        <v>42</v>
+      </c>
+      <c r="G2" s="20">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="19" t="s">
+        <v>65</v>
+      </c>
+      <c r="B3" s="20">
+        <v>47</v>
+      </c>
+      <c r="C3" s="21">
+        <v>0.104</v>
+      </c>
+      <c r="E3" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" s="20">
+        <v>90</v>
+      </c>
+      <c r="G3" s="20">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="20">
+        <v>58</v>
+      </c>
+      <c r="C4" s="21">
+        <v>0.128</v>
+      </c>
+      <c r="E4" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="F4" s="20">
+        <v>161</v>
+      </c>
+      <c r="G4" s="20">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="B5" s="20">
+        <v>83</v>
+      </c>
+      <c r="C5" s="21">
+        <v>0.183</v>
+      </c>
+      <c r="E5" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="F5" s="20">
+        <v>247</v>
+      </c>
+      <c r="G5" s="20">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="20">
+        <v>104</v>
+      </c>
+      <c r="C6" s="21">
+        <v>0.229</v>
+      </c>
+      <c r="E6" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="F6" s="20">
+        <v>284</v>
+      </c>
+      <c r="G6" s="20">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="19" t="s">
+        <v>67</v>
+      </c>
+      <c r="B7" s="20">
+        <v>134</v>
+      </c>
+      <c r="C7" s="21">
+        <v>0.295</v>
+      </c>
+      <c r="E7" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="F7" s="20">
+        <v>321</v>
+      </c>
+      <c r="G7" s="20">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="E10" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="F10" s="18" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="B11" s="21">
+        <v>0.39</v>
+      </c>
+      <c r="E11" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="F11" s="20">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="B12" s="21">
+        <v>0.3</v>
+      </c>
+      <c r="E12" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="F12" s="20">
         <v>55</v>
       </c>
-      <c r="B1" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="C1" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="E1" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="F1" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="G1" s="15" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="16" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" s="17">
-        <v>28</v>
-      </c>
-      <c r="C2" s="18">
-        <v>0.062</v>
-      </c>
-      <c r="E2" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F2" s="17">
-        <v>42</v>
-      </c>
-      <c r="G2" s="17">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="B3" s="17">
-        <v>47</v>
-      </c>
-      <c r="C3" s="18">
-        <v>0.104</v>
-      </c>
-      <c r="E3" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="F3" s="17">
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="B13" s="21">
+        <v>0.29</v>
+      </c>
+      <c r="E13" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="F13" s="20">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="21">
+        <v>0.25</v>
+      </c>
+      <c r="E14" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="F14" s="20">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="B15" s="21">
+        <v>0.12</v>
+      </c>
+      <c r="E15" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="F15" s="20">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="B16" s="21">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="18" t="s">
+        <v>84</v>
+      </c>
+      <c r="B18" s="18" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="B19" s="20">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="B20" s="20">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="B21" s="20">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="B22" s="20">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="G3" s="17">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" s="17">
-        <v>58</v>
-      </c>
-      <c r="C4" s="18">
-        <v>0.128</v>
-      </c>
-      <c r="E4" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="F4" s="17">
-        <v>161</v>
-      </c>
-      <c r="G4" s="17">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="B5" s="17">
-        <v>83</v>
-      </c>
-      <c r="C5" s="18">
-        <v>0.183</v>
-      </c>
-      <c r="E5" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="F5" s="17">
-        <v>247</v>
-      </c>
-      <c r="G5" s="17">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="17">
-        <v>104</v>
-      </c>
-      <c r="C6" s="18">
-        <v>0.229</v>
-      </c>
-      <c r="E6" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="F6" s="17">
-        <v>284</v>
-      </c>
-      <c r="G6" s="17">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="B7" s="17">
-        <v>134</v>
-      </c>
-      <c r="C7" s="18">
-        <v>0.295</v>
-      </c>
-      <c r="E7" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="F7" s="17">
-        <v>321</v>
-      </c>
-      <c r="G7" s="17">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="A10" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="B10" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="E10" s="15" t="s">
+      <c r="B23" s="20">
         <v>70</v>
       </c>
-      <c r="F10" s="15" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="A11" s="16" t="s">
-        <v>65</v>
-      </c>
-      <c r="B11" s="18">
-        <v>0.39</v>
-      </c>
-      <c r="E11" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="F11" s="17">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="A12" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="B12" s="18">
-        <v>0.3</v>
-      </c>
-      <c r="E12" s="16" t="s">
-        <v>73</v>
-      </c>
-      <c r="F12" s="17">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="A13" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="B13" s="18">
-        <v>0.29</v>
-      </c>
-      <c r="E13" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="F13" s="17">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
-      <c r="A14" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" s="18">
-        <v>0.25</v>
-      </c>
-      <c r="E14" s="16" t="s">
-        <v>75</v>
-      </c>
-      <c r="F14" s="17">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
-      <c r="A15" s="16" t="s">
-        <v>68</v>
-      </c>
-      <c r="B15" s="18">
-        <v>0.12</v>
-      </c>
-      <c r="E15" s="16" t="s">
-        <v>76</v>
-      </c>
-      <c r="F15" s="17">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
-      <c r="A16" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="B16" s="18">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2">
-      <c r="A18" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="B18" s="15" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2">
-      <c r="A19" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="B19" s="17">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2">
-      <c r="A20" s="16" t="s">
-        <v>80</v>
-      </c>
-      <c r="B20" s="17">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2">
-      <c r="A21" s="16" t="s">
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="B24" s="20">
         <v>81</v>
       </c>
-      <c r="B21" s="17">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2">
-      <c r="A22" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="B22" s="17">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2">
-      <c r="A23" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="B23" s="17">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2">
-      <c r="A24" s="16" t="s">
-        <v>84</v>
-      </c>
-      <c r="B24" s="17">
-        <v>81</v>
-      </c>
     </row>
     <row r="25" spans="1:2">
-      <c r="A25" s="16" t="s">
-        <v>85</v>
-      </c>
-      <c r="B25" s="17">
+      <c r="A25" s="19" t="s">
+        <v>92</v>
+      </c>
+      <c r="B25" s="20">
         <v>82</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Add Target Progress Bars, Scorecards and Egyptian Hubs to Excel Dashboard
</commit_message>
<xml_diff>
--- a/Shark_Gym_Workforce_Dashboard.xlsx
+++ b/Shark_Gym_Workforce_Dashboard.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="102">
   <si>
     <t>🦈 SHARK GYM</t>
   </si>
@@ -208,6 +208,45 @@
 • Gender Floor Parity: Maintain current 60% M / 40% F ratio across all morning and evening shifts.</t>
   </si>
   <si>
+    <t>4. MONTHLY TARGET PROGRESS &amp; KPI SCORECARDS (EGP)</t>
+  </si>
+  <si>
+    <t>🏆 Monthly PT Revenue Target (EGP 2.0M)</t>
+  </si>
+  <si>
+    <t>█████████░  EGP 1,820,000 Actual</t>
+  </si>
+  <si>
+    <t>91.0% Achieved</t>
+  </si>
+  <si>
+    <t>🏋️ Master Coach Hiring Target (35 Coaches)</t>
+  </si>
+  <si>
+    <t>██████████  34 Coaches Onboarded</t>
+  </si>
+  <si>
+    <t>97.1% Achieved</t>
+  </si>
+  <si>
+    <t>⚡ Floor Shift Biometric Compliance (95%)</t>
+  </si>
+  <si>
+    <t>██████████  98.7% Punch-in Rate</t>
+  </si>
+  <si>
+    <t>103.9% Benchmark</t>
+  </si>
+  <si>
+    <t>🛡️ Member Retention Index (Target 80%)</t>
+  </si>
+  <si>
+    <t>█████████░  86.5% Active Athletes</t>
+  </si>
+  <si>
+    <t>+6.5% Surplus</t>
+  </si>
+  <si>
     <t>Department</t>
   </si>
   <si>
@@ -280,25 +319,13 @@
     <t>Staff Count</t>
   </si>
   <si>
-    <t>Gurugram / Tagamoa</t>
-  </si>
-  <si>
-    <t>Mumbai / Zayed</t>
-  </si>
-  <si>
-    <t>Hyderabad / Degla</t>
-  </si>
-  <si>
-    <t>Chennai / Korba</t>
-  </si>
-  <si>
-    <t>Pune Hub</t>
-  </si>
-  <si>
-    <t>Bengaluru Hub</t>
-  </si>
-  <si>
-    <t>Delhi Compound</t>
+    <t>6th October Arena</t>
+  </si>
+  <si>
+    <t>Alexandria Flagship</t>
+  </si>
+  <si>
+    <t>Katameya Heights</t>
   </si>
 </sst>
 </file>
@@ -309,7 +336,7 @@
     <numFmt numFmtId="164" formatCode="#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -419,13 +446,34 @@
       <family val="2"/>
     </font>
     <font>
+      <b/>
+      <sz val="9.5"/>
+      <color rgb="FF2A1147"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9.5"/>
+      <color rgb="FF166534"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9.5"/>
+      <color rgb="FF4A1572"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="9"/>
       <color theme="1"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -468,8 +516,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF3E8FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCFCE7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -559,6 +619,21 @@
     </border>
     <border>
       <left style="thin">
+        <color rgb="FF86EFAC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF86EFAC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF86EFAC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF86EFAC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color rgb="FF2E0A4F"/>
       </left>
       <right style="thin">
@@ -591,7 +666,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -642,12 +717,21 @@
     <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -1649,25 +1733,25 @@
               <c:strCache>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>Gurugram / Tagamoa</c:v>
+                  <c:v>New Cairo (Tagamoa)</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Mumbai / Zayed</c:v>
+                  <c:v>Sheikh Zayed (Arkan)</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Hyderabad / Degla</c:v>
+                  <c:v>Maadi (Degla)</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Chennai / Korba</c:v>
+                  <c:v>Heliopolis (Korba)</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Pune Hub</c:v>
+                  <c:v>6th October Arena</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Bengaluru Hub</c:v>
+                  <c:v>Alexandria Flagship</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Delhi Compound</c:v>
+                  <c:v>Katameya Heights</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1679,25 +1763,25 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>53</c:v>
+                  <c:v>92</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>84</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>76</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>68</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>54</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>54</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>60</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>70</c:v>
-                </c:pt>
                 <c:pt idx="5">
-                  <c:v>81</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>82</c:v>
+                  <c:v>32</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2764,52 +2848,103 @@
       <c r="G16" s="17"/>
       <c r="H16" s="17"/>
     </row>
-    <row r="17" spans="2:2">
+    <row r="17" spans="2:8">
       <c r="B17" s="6"/>
     </row>
-    <row r="18" spans="2:2">
+    <row r="18" spans="2:8">
       <c r="B18" s="6"/>
-    </row>
-    <row r="19" spans="2:2">
+      <c r="D18" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+    </row>
+    <row r="19" spans="2:8">
       <c r="B19" s="6"/>
-    </row>
-    <row r="20" spans="2:2">
+      <c r="D19" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="E19" s="18"/>
+      <c r="F19" s="19" t="s">
+        <v>64</v>
+      </c>
+      <c r="G19" s="19"/>
+      <c r="H19" s="20" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8">
       <c r="B20" s="6"/>
-    </row>
-    <row r="21" spans="2:2">
+      <c r="D20" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="E20" s="18"/>
+      <c r="F20" s="19" t="s">
+        <v>67</v>
+      </c>
+      <c r="G20" s="19"/>
+      <c r="H20" s="20" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8">
       <c r="B21" s="6"/>
-    </row>
-    <row r="22" spans="2:2">
+      <c r="D21" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="E21" s="18"/>
+      <c r="F21" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="G21" s="19"/>
+      <c r="H21" s="20" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8">
       <c r="B22" s="6"/>
-    </row>
-    <row r="23" spans="2:2">
+      <c r="D22" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="E22" s="18"/>
+      <c r="F22" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="G22" s="19"/>
+      <c r="H22" s="20" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="23" spans="2:8">
       <c r="B23" s="6"/>
     </row>
-    <row r="24" spans="2:2">
+    <row r="24" spans="2:8">
       <c r="B24" s="6"/>
     </row>
-    <row r="25" spans="2:2">
+    <row r="25" spans="2:8">
       <c r="B25" s="6"/>
     </row>
-    <row r="26" spans="2:2">
+    <row r="26" spans="2:8">
       <c r="B26" s="6"/>
     </row>
-    <row r="27" spans="2:2">
+    <row r="27" spans="2:8">
       <c r="B27" s="6"/>
     </row>
-    <row r="28" spans="2:2">
+    <row r="28" spans="2:8">
       <c r="B28" s="6"/>
     </row>
-    <row r="29" spans="2:2">
+    <row r="29" spans="2:8">
       <c r="B29" s="6"/>
     </row>
-    <row r="30" spans="2:2">
+    <row r="30" spans="2:8">
       <c r="B30" s="6"/>
     </row>
-    <row r="31" spans="2:2">
+    <row r="31" spans="2:8">
       <c r="B31" s="6"/>
     </row>
-    <row r="32" spans="2:2">
+    <row r="32" spans="2:8">
       <c r="B32" s="6"/>
     </row>
     <row r="33" spans="2:2">
@@ -2822,7 +2957,7 @@
       <c r="B35" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="16">
     <mergeCell ref="D2:H2"/>
     <mergeCell ref="D4:H4"/>
     <mergeCell ref="D5:H6"/>
@@ -2830,6 +2965,15 @@
     <mergeCell ref="D9:H11"/>
     <mergeCell ref="D13:H13"/>
     <mergeCell ref="D14:H16"/>
+    <mergeCell ref="D18:H18"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="F22:G22"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B7" location="Dashboard!A1" display="📊  Dashboard"/>
@@ -2850,299 +2994,299 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="B1" s="18" t="s">
-        <v>63</v>
-      </c>
-      <c r="C1" s="18" t="s">
-        <v>64</v>
-      </c>
-      <c r="E1" s="18" t="s">
+      <c r="A1" s="21" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="E1" s="21" t="s">
+        <v>81</v>
+      </c>
+      <c r="F1" s="21" t="s">
+        <v>82</v>
+      </c>
+      <c r="G1" s="21" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="23">
+        <v>28</v>
+      </c>
+      <c r="C2" s="24">
+        <v>0.062</v>
+      </c>
+      <c r="E2" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="F2" s="23">
+        <v>42</v>
+      </c>
+      <c r="G2" s="23">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3" s="23">
+        <v>47</v>
+      </c>
+      <c r="C3" s="24">
+        <v>0.104</v>
+      </c>
+      <c r="E3" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" s="23">
+        <v>90</v>
+      </c>
+      <c r="G3" s="23">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="23">
+        <v>58</v>
+      </c>
+      <c r="C4" s="24">
+        <v>0.128</v>
+      </c>
+      <c r="E4" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="F4" s="23">
+        <v>161</v>
+      </c>
+      <c r="G4" s="23">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" s="23">
+        <v>83</v>
+      </c>
+      <c r="C5" s="24">
+        <v>0.183</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="F5" s="23">
+        <v>247</v>
+      </c>
+      <c r="G5" s="23">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="23">
+        <v>104</v>
+      </c>
+      <c r="C6" s="24">
+        <v>0.229</v>
+      </c>
+      <c r="E6" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="F6" s="23">
+        <v>284</v>
+      </c>
+      <c r="G6" s="23">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="22" t="s">
+        <v>80</v>
+      </c>
+      <c r="B7" s="23">
+        <v>134</v>
+      </c>
+      <c r="C7" s="24">
+        <v>0.295</v>
+      </c>
+      <c r="E7" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="F7" s="23">
+        <v>321</v>
+      </c>
+      <c r="G7" s="23">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="21" t="s">
+        <v>75</v>
+      </c>
+      <c r="B10" s="21" t="s">
+        <v>84</v>
+      </c>
+      <c r="E10" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="F10" s="21" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="B11" s="24">
+        <v>0.39</v>
+      </c>
+      <c r="E11" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="F11" s="23">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="B12" s="24">
+        <v>0.3</v>
+      </c>
+      <c r="E12" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="F12" s="23">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="B13" s="24">
+        <v>0.29</v>
+      </c>
+      <c r="E13" s="22" t="s">
+        <v>94</v>
+      </c>
+      <c r="F13" s="23">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="24">
+        <v>0.25</v>
+      </c>
+      <c r="E14" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="F14" s="23">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" s="22" t="s">
+        <v>88</v>
+      </c>
+      <c r="B15" s="24">
+        <v>0.12</v>
+      </c>
+      <c r="E15" s="22" t="s">
+        <v>96</v>
+      </c>
+      <c r="F15" s="23">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="B16" s="24">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="B18" s="21" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" s="23">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20" s="23">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="23">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="23">
         <v>68</v>
       </c>
-      <c r="F1" s="18" t="s">
-        <v>69</v>
-      </c>
-      <c r="G1" s="18" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" s="20">
-        <v>28</v>
-      </c>
-      <c r="C2" s="21">
-        <v>0.062</v>
-      </c>
-      <c r="E2" s="19" t="s">
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" s="22" t="s">
+        <v>99</v>
+      </c>
+      <c r="B23" s="23">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" s="22" t="s">
+        <v>100</v>
+      </c>
+      <c r="B24" s="23">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" s="22" t="s">
+        <v>101</v>
+      </c>
+      <c r="B25" s="23">
         <v>32</v>
-      </c>
-      <c r="F2" s="20">
-        <v>42</v>
-      </c>
-      <c r="G2" s="20">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="19" t="s">
-        <v>65</v>
-      </c>
-      <c r="B3" s="20">
-        <v>47</v>
-      </c>
-      <c r="C3" s="21">
-        <v>0.104</v>
-      </c>
-      <c r="E3" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="F3" s="20">
-        <v>90</v>
-      </c>
-      <c r="G3" s="20">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="19" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" s="20">
-        <v>58</v>
-      </c>
-      <c r="C4" s="21">
-        <v>0.128</v>
-      </c>
-      <c r="E4" s="19" t="s">
-        <v>34</v>
-      </c>
-      <c r="F4" s="20">
-        <v>161</v>
-      </c>
-      <c r="G4" s="20">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="19" t="s">
-        <v>66</v>
-      </c>
-      <c r="B5" s="20">
-        <v>83</v>
-      </c>
-      <c r="C5" s="21">
-        <v>0.183</v>
-      </c>
-      <c r="E5" s="19" t="s">
-        <v>35</v>
-      </c>
-      <c r="F5" s="20">
-        <v>247</v>
-      </c>
-      <c r="G5" s="20">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="20">
-        <v>104</v>
-      </c>
-      <c r="C6" s="21">
-        <v>0.229</v>
-      </c>
-      <c r="E6" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="F6" s="20">
-        <v>284</v>
-      </c>
-      <c r="G6" s="20">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="19" t="s">
-        <v>67</v>
-      </c>
-      <c r="B7" s="20">
-        <v>134</v>
-      </c>
-      <c r="C7" s="21">
-        <v>0.295</v>
-      </c>
-      <c r="E7" s="19" t="s">
-        <v>37</v>
-      </c>
-      <c r="F7" s="20">
-        <v>321</v>
-      </c>
-      <c r="G7" s="20">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="A10" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="B10" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="E10" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="F10" s="18" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="A11" s="19" t="s">
-        <v>72</v>
-      </c>
-      <c r="B11" s="21">
-        <v>0.39</v>
-      </c>
-      <c r="E11" s="19" t="s">
-        <v>79</v>
-      </c>
-      <c r="F11" s="20">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="A12" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="B12" s="21">
-        <v>0.3</v>
-      </c>
-      <c r="E12" s="19" t="s">
-        <v>80</v>
-      </c>
-      <c r="F12" s="20">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="A13" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="B13" s="21">
-        <v>0.29</v>
-      </c>
-      <c r="E13" s="19" t="s">
-        <v>81</v>
-      </c>
-      <c r="F13" s="20">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
-      <c r="A14" s="19" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" s="21">
-        <v>0.25</v>
-      </c>
-      <c r="E14" s="19" t="s">
-        <v>82</v>
-      </c>
-      <c r="F14" s="20">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
-      <c r="A15" s="19" t="s">
-        <v>75</v>
-      </c>
-      <c r="B15" s="21">
-        <v>0.12</v>
-      </c>
-      <c r="E15" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="F15" s="20">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
-      <c r="A16" s="19" t="s">
-        <v>76</v>
-      </c>
-      <c r="B16" s="21">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2">
-      <c r="A18" s="18" t="s">
-        <v>84</v>
-      </c>
-      <c r="B18" s="18" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2">
-      <c r="A19" s="19" t="s">
-        <v>86</v>
-      </c>
-      <c r="B19" s="20">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2">
-      <c r="A20" s="19" t="s">
-        <v>87</v>
-      </c>
-      <c r="B20" s="20">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2">
-      <c r="A21" s="19" t="s">
-        <v>88</v>
-      </c>
-      <c r="B21" s="20">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2">
-      <c r="A22" s="19" t="s">
-        <v>89</v>
-      </c>
-      <c r="B22" s="20">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2">
-      <c r="A23" s="19" t="s">
-        <v>90</v>
-      </c>
-      <c r="B23" s="20">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2">
-      <c r="A24" s="19" t="s">
-        <v>91</v>
-      </c>
-      <c r="B24" s="20">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2">
-      <c r="A25" s="19" t="s">
-        <v>92</v>
-      </c>
-      <c r="B25" s="20">
-        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Add Pro suite - Web Audio API synthesizer, TV Wallboard mode, Live search drawer, KPI sparklines, and Excel Payroll Simulator
</commit_message>
<xml_diff>
--- a/Shark_Gym_Workforce_Dashboard.xlsx
+++ b/Shark_Gym_Workforce_Dashboard.xlsx
@@ -7,16 +7,18 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" r:id="rId2"/>
-    <sheet name="Data_Engine" sheetId="3" r:id="rId3"/>
+    <sheet name="Welcome_HQ" sheetId="1" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" r:id="rId2"/>
+    <sheet name="Summary" sheetId="3" r:id="rId3"/>
+    <sheet name="Payroll_Simulator" sheetId="4" r:id="rId4"/>
+    <sheet name="Data_Engine" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="139">
   <si>
     <t>🦈 SHARK GYM</t>
   </si>
@@ -24,19 +26,73 @@
     <t>WORKFORCE INTELLIGENCE</t>
   </si>
   <si>
+    <t>🏛️  HQ Cover</t>
+  </si>
+  <si>
     <t>📊  Dashboard</t>
   </si>
   <si>
-    <t>📈  Summary</t>
-  </si>
-  <si>
-    <t>🗄️  Database</t>
-  </si>
-  <si>
-    <t>⚜️ ATHLETIC HQ</t>
-  </si>
-  <si>
-    <t>CAIRO • EGYPT</t>
+    <t>📈  Summary Memo</t>
+  </si>
+  <si>
+    <t>💰  Payroll Simulator</t>
+  </si>
+  <si>
+    <t>🗄️  Data Engine</t>
+  </si>
+  <si>
+    <t>🦈 SHARK GYM ATHLETIC ENTERPRISE</t>
+  </si>
+  <si>
+    <t>Executive Workforce Analytics, Staffing &amp; Payroll Simulator (EGP)</t>
+  </si>
+  <si>
+    <t>EXECUTIVE BRIEFING &amp; DOCUMENT METADATA</t>
+  </si>
+  <si>
+    <t>Enterprise Entity:</t>
+  </si>
+  <si>
+    <t>Shark Gym Egyptian Athletic Compounds (Cairo / Giza / Alex / Delta)</t>
+  </si>
+  <si>
+    <t>Reporting Fiscal Period:</t>
+  </si>
+  <si>
+    <t>Fiscal Year 2026 Live Performance &amp; Staffing Velocity</t>
+  </si>
+  <si>
+    <t>Base Operating Currency:</t>
+  </si>
+  <si>
+    <t>Egyptian Pounds (L.E / EGP) — All Compensation &amp; Revenue Models</t>
+  </si>
+  <si>
+    <t>Audit &amp; Biometric Sync:</t>
+  </si>
+  <si>
+    <t>100% Shift Attendance Sync via Integrated Biometric Readers</t>
+  </si>
+  <si>
+    <t>Classification:</t>
+  </si>
+  <si>
+    <t>Boardroom Executive Confidential — Workforce Intelligence HQ</t>
+  </si>
+  <si>
+    <t>DIRECT INTERACTIVE JUMP LINKS</t>
+  </si>
+  <si>
+    <t>📊  Open Master Dashboard</t>
+  </si>
+  <si>
+    <t>📈  Executive Board Memo</t>
+  </si>
+  <si>
+    <t>💰  Open Payroll Calculator</t>
+  </si>
+  <si>
+    <t>🗄️  Inspect Raw Data</t>
   </si>
   <si>
     <t xml:space="preserve">  📊 Employee WorkForce Dashboard</t>
@@ -97,15 +153,6 @@
   </si>
   <si>
     <t>Fiscal Year ▾</t>
-  </si>
-  <si>
-    <t>2023</t>
-  </si>
-  <si>
-    <t>2024</t>
-  </si>
-  <si>
-    <t>2025</t>
   </si>
   <si>
     <t>2026 (Live)</t>
@@ -197,7 +244,7 @@
   <si>
     <t>• Strength &amp; Conditioning: Lowest attrition in compound history (8%), with 134 certified barbell coaches.
 • High Average Tenure: 5.1 years average retention among Master Coaches (L3), ensuring training quality.
-• Cairo Hub Density: New Cairo leads with 82 coaches, followed closely by Sheikh Zayed at 81 coaches.</t>
+• Cairo Hub Density: New Cairo leads with 92 coaches, followed closely by Sheikh Zayed at 84 coaches.</t>
   </si>
   <si>
     <t>3. OPERATIONAL ACTION ITEMS &amp; INCENTIVES (EGP)</t>
@@ -245,6 +292,72 @@
   </si>
   <si>
     <t>+6.5% Surplus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  💰 Coach Compensation &amp; VIP Session Revenue Simulator (EGP)</t>
+  </si>
+  <si>
+    <t>Coach Name</t>
+  </si>
+  <si>
+    <t>Compound Hub</t>
+  </si>
+  <si>
+    <t>Base Salary</t>
+  </si>
+  <si>
+    <t>PT Sessions</t>
+  </si>
+  <si>
+    <t>Session Rate</t>
+  </si>
+  <si>
+    <t>PT Revenue</t>
+  </si>
+  <si>
+    <t>Gym Margin (40%)</t>
+  </si>
+  <si>
+    <t>Net Coach Payout</t>
+  </si>
+  <si>
+    <t>Sherif El-Bendary</t>
+  </si>
+  <si>
+    <t>New Cairo</t>
+  </si>
+  <si>
+    <t>Dr. Nourhan Tarek</t>
+  </si>
+  <si>
+    <t>Maadi Degla</t>
+  </si>
+  <si>
+    <t>Tamer Hosny</t>
+  </si>
+  <si>
+    <t>Sheikh Zayed</t>
+  </si>
+  <si>
+    <t>Ahmed Zaki</t>
+  </si>
+  <si>
+    <t>Heliopolis</t>
+  </si>
+  <si>
+    <t>Mariam Mansour</t>
+  </si>
+  <si>
+    <t>Karim Hegazy</t>
+  </si>
+  <si>
+    <t>6th October</t>
+  </si>
+  <si>
+    <t>TOTALS &amp; MONTHLY ACCRUAL</t>
+  </si>
+  <si>
+    <t>AVG / BLENDED</t>
   </si>
   <si>
     <t>Department</t>
@@ -332,11 +445,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="#,##0"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="&quot;EGP &quot;#,##0"/>
+    <numFmt numFmtId="165" formatCode="#,##0"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -353,8 +467,61 @@
     </font>
     <font>
       <b/>
+      <sz val="24"/>
+      <color rgb="FFF59E0B"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8.5"/>
+      <color rgb="FFF59E0B"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFE9D5FF"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10.5"/>
+      <color rgb="FF3E1C66"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF4A1572"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF2A1147"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFE9D5FF"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
       <sz val="16"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF2A0E4F"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
@@ -366,34 +533,21 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="8"/>
-      <color rgb="FFD1B8F0"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-    </font>
-    <font>
+      <i/>
       <sz val="9"/>
-      <color rgb="FFDCC9F5"/>
+      <color rgb="FF6B21A8"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
-      <color rgb="FF4A1572"/>
+      <color rgb="FF3E1C66"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="8.5"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color rgb="FF4A1572"/>
       <name val="Segoe UI"/>
       <family val="2"/>
@@ -401,40 +555,26 @@
     <font>
       <b/>
       <sz val="8.5"/>
-      <color rgb="FF756285"/>
+      <color rgb="FF5A228F"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="10"/>
-      <color rgb="FFE0D1F7"/>
+      <sz val="18"/>
+      <color rgb="FF2A0E4F"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF68239E"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="20"/>
-      <color rgb="FF4A1572"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <color rgb="FF9E8FB0"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color rgb="FF8E6BB8"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="16"/>
       <color rgb="FFFFFFFF"/>
       <name val="Segoe UI"/>
       <family val="2"/>
@@ -473,7 +613,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -488,13 +628,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEDE4F7"/>
+        <fgColor rgb="FF5A228F"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF682A99"/>
+        <fgColor rgb="FFF7F3FB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF3E8FF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -506,19 +652,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF4A1572"/>
+        <fgColor rgb="FF68239E"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF5A228F"/>
+        <fgColor rgb="FFF0E6F7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF3E8FF"/>
+        <fgColor rgb="FFFCFAFF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -529,12 +675,25 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="13">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF9333EA"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD5C4EA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD5C4EA"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -554,29 +713,55 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF501F7A"/>
+        <color rgb="FFA855F7"/>
       </left>
       <right style="thin">
-        <color rgb="FF501F7A"/>
+        <color rgb="FFA855F7"/>
       </right>
       <top style="thin">
-        <color rgb="FF501F7A"/>
+        <color rgb="FFA855F7"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF501F7A"/>
+        <color rgb="FFA855F7"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color rgb="FFBDA1E5"/>
+      <left style="thin">
+        <color rgb="FF5A2283"/>
       </left>
-      <right/>
+      <right style="thin">
+        <color rgb="FF5A2283"/>
+      </right>
       <top style="thin">
-        <color rgb="FFD5C4EA"/>
+        <color rgb="FF5A2283"/>
       </top>
       <bottom style="thin">
+        <color rgb="FF5A2283"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
         <color rgb="FFD5C4EA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE0D2EF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE0D2EF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE0D2EF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE0D2EF"/>
       </bottom>
       <diagonal/>
     </border>
@@ -666,73 +851,92 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="165" fontId="23" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="19" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="166" fontId="23" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1691,7 +1895,7 @@
                   <a:srgbClr val="2A0E4F"/>
                 </a:solidFill>
               </a:rPr>
-              <a:t>Employees by Location</a:t>
+              <a:t>Employees by Location (Egyptian Compounds)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1878,7 +2082,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>66675</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>24</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -1907,8 +2111,8 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>219075</xdr:colOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>24</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -1968,7 +2172,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>66675</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>37</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -1997,8 +2201,8 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>219075</xdr:colOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>37</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -2310,358 +2514,608 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="B2:G40"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="3.7109375" customWidth="1"/>
+    <col min="2" max="2" width="24.7109375" customWidth="1"/>
+    <col min="3" max="3" width="3.7109375" customWidth="1"/>
+    <col min="4" max="7" width="22.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:7">
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+    </row>
+    <row r="3" spans="2:7">
+      <c r="B3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+    </row>
+    <row r="4" spans="2:7">
+      <c r="B4" s="4"/>
+      <c r="D4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+    </row>
+    <row r="5" spans="2:7">
+      <c r="B5" s="4"/>
+    </row>
+    <row r="6" spans="2:7">
+      <c r="B6" s="4"/>
+      <c r="D6" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+    </row>
+    <row r="7" spans="2:7">
+      <c r="B7" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+    </row>
+    <row r="8" spans="2:7">
+      <c r="B8" s="4"/>
+      <c r="D8" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+    </row>
+    <row r="9" spans="2:7">
+      <c r="B9" s="4"/>
+      <c r="D9" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+    </row>
+    <row r="10" spans="2:7">
+      <c r="B10" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+    </row>
+    <row r="11" spans="2:7">
+      <c r="B11" s="4"/>
+      <c r="D11" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+    </row>
+    <row r="12" spans="2:7">
+      <c r="B12" s="4"/>
+    </row>
+    <row r="13" spans="2:7">
+      <c r="B13" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+    </row>
+    <row r="14" spans="2:7">
+      <c r="B14" s="4"/>
+    </row>
+    <row r="15" spans="2:7">
+      <c r="B15" s="4"/>
+      <c r="D15" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7">
+      <c r="B16" s="10" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2">
+      <c r="B17" s="4"/>
+    </row>
+    <row r="18" spans="2:2">
+      <c r="B18" s="4"/>
+    </row>
+    <row r="19" spans="2:2">
+      <c r="B19" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2">
+      <c r="B20" s="4"/>
+    </row>
+    <row r="21" spans="2:2">
+      <c r="B21" s="4"/>
+    </row>
+    <row r="22" spans="2:2">
+      <c r="B22" s="4"/>
+    </row>
+    <row r="23" spans="2:2">
+      <c r="B23" s="4"/>
+    </row>
+    <row r="24" spans="2:2">
+      <c r="B24" s="4"/>
+    </row>
+    <row r="25" spans="2:2">
+      <c r="B25" s="4"/>
+    </row>
+    <row r="26" spans="2:2">
+      <c r="B26" s="4"/>
+    </row>
+    <row r="27" spans="2:2">
+      <c r="B27" s="4"/>
+    </row>
+    <row r="28" spans="2:2">
+      <c r="B28" s="4"/>
+    </row>
+    <row r="29" spans="2:2">
+      <c r="B29" s="4"/>
+    </row>
+    <row r="30" spans="2:2">
+      <c r="B30" s="4"/>
+    </row>
+    <row r="31" spans="2:2">
+      <c r="B31" s="4"/>
+    </row>
+    <row r="32" spans="2:2">
+      <c r="B32" s="4"/>
+    </row>
+    <row r="33" spans="2:2">
+      <c r="B33" s="4"/>
+    </row>
+    <row r="34" spans="2:2">
+      <c r="B34" s="4"/>
+    </row>
+    <row r="35" spans="2:2">
+      <c r="B35" s="4"/>
+    </row>
+    <row r="36" spans="2:2">
+      <c r="B36" s="4"/>
+    </row>
+    <row r="37" spans="2:2">
+      <c r="B37" s="4"/>
+    </row>
+    <row r="38" spans="2:2">
+      <c r="B38" s="4"/>
+    </row>
+    <row r="39" spans="2:2">
+      <c r="B39" s="4"/>
+    </row>
+    <row r="40" spans="2:2">
+      <c r="B40" s="4"/>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="D2:G3"/>
+    <mergeCell ref="D4:G4"/>
+    <mergeCell ref="D6:G6"/>
+    <mergeCell ref="E7:G7"/>
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="E9:G9"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="D13:G13"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="B7" location="Welcome_HQ!A1" display="🏛️  HQ Cover"/>
+    <hyperlink ref="B10" location="Dashboard!A1" display="📊  Dashboard"/>
+    <hyperlink ref="B13" location="Summary!A1" display="📈  Summary Memo"/>
+    <hyperlink ref="D15" location="Dashboard!A1" display="📊  Open Master Dashboard"/>
+    <hyperlink ref="E15" location="Summary!A1" display="📈  Executive Board Memo"/>
+    <hyperlink ref="F15" location="Payroll_Simulator!A1" display="💰  Open Payroll Calculator"/>
+    <hyperlink ref="G15" location="Data_Engine!A1" display="🗄️  Inspect Raw Data"/>
+    <hyperlink ref="B16" location="Payroll_Simulator!A1" display="💰  Payroll Simulator"/>
+    <hyperlink ref="B19" location="Data_Engine!A1" display="🗄️  Data Engine"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup fitToHeight="0" orientation="landscape"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A2:O44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="2.7109375" customWidth="1"/>
     <col min="2" max="2" width="22.7109375" customWidth="1"/>
     <col min="3" max="3" width="2.7109375" customWidth="1"/>
-    <col min="4" max="9" width="15.7109375" customWidth="1"/>
-    <col min="10" max="11" width="14.7109375" customWidth="1"/>
-    <col min="12" max="15" width="10.28515625" customWidth="1"/>
-    <col min="16" max="16" width="2.7109375" customWidth="1"/>
+    <col min="4" max="15" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" ht="26" customHeight="1">
+    <row r="2" spans="2:15" ht="28" customHeight="1">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="O2" s="3"/>
+      <c r="D2" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="O2" s="13"/>
     </row>
     <row r="3" spans="2:15" ht="18" customHeight="1">
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
-      <c r="L3" s="5"/>
-      <c r="M3" s="5"/>
-      <c r="N3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="O3" s="3"/>
+      <c r="D3" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="14"/>
+      <c r="L3" s="14"/>
+      <c r="M3" s="14"/>
+      <c r="N3" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="O3" s="13"/>
     </row>
     <row r="4" spans="2:15">
-      <c r="B4" s="6"/>
+      <c r="B4" s="4"/>
     </row>
     <row r="5" spans="2:15" ht="20" customHeight="1">
-      <c r="B5" s="6"/>
-      <c r="D5" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="K5" s="7"/>
-      <c r="L5" s="7" t="s">
+      <c r="B5" s="4"/>
+      <c r="D5" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="K5" s="15"/>
+      <c r="L5" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="M5" s="15"/>
+      <c r="N5" s="15"/>
+      <c r="O5" s="15"/>
+    </row>
+    <row r="6" spans="2:15" ht="20" customHeight="1">
+      <c r="B6" s="4"/>
+      <c r="D6" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="M5" s="7"/>
-      <c r="N5" s="7"/>
-      <c r="O5" s="7"/>
-    </row>
-    <row r="6" spans="2:15" ht="20" customHeight="1">
-      <c r="B6" s="6"/>
-      <c r="D6" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="H6" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="I6" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="J6" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="K6" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="L6" s="8" t="s">
+      <c r="F6" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="G6" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="H6" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="I6" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="J6" s="16">
+        <v>2023</v>
+      </c>
+      <c r="K6" s="16">
+        <v>2024</v>
+      </c>
+      <c r="L6" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="M6" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="N6" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="O6" s="16" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="2:15" ht="20" customHeight="1">
+      <c r="B7" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="M6" s="8" t="s">
+      <c r="E7" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="N6" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="O6" s="8" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7" spans="2:15" ht="20" customHeight="1">
-      <c r="B7" s="9" t="s">
-        <v>2</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="H7" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="I7" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="J7" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="K7" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="L7" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="M7" s="8" t="s">
+      <c r="F7" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="N7" s="8" t="s">
+      <c r="G7" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="O7" s="8" t="s">
-        <v>39</v>
+      <c r="H7" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="I7" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="J7" s="16">
+        <v>2025</v>
+      </c>
+      <c r="K7" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="L7" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M7" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="N7" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="O7" s="16" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="2:15">
-      <c r="B8" s="6"/>
+      <c r="B8" s="4"/>
     </row>
     <row r="9" spans="2:15" ht="18" customHeight="1">
-      <c r="B9" s="6"/>
-      <c r="D9" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="I9" s="10"/>
-      <c r="J9" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="K9" s="10"/>
-      <c r="L9" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="M9" s="10"/>
-      <c r="N9" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="O9" s="10"/>
+      <c r="B9" s="4"/>
+      <c r="D9" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="K9" s="17"/>
+      <c r="L9" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="M9" s="17"/>
+      <c r="N9" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="O9" s="17"/>
     </row>
     <row r="10" spans="2:15" ht="30" customHeight="1">
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="D10" s="12">
+      <c r="D10" s="18">
         <v>454</v>
       </c>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12">
+      <c r="E10" s="18"/>
+      <c r="F10" s="18">
         <v>321</v>
       </c>
-      <c r="G10" s="12"/>
-      <c r="H10" s="12">
+      <c r="G10" s="18"/>
+      <c r="H10" s="18">
         <v>133</v>
       </c>
-      <c r="I10" s="12"/>
-      <c r="J10" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="K10" s="12"/>
-      <c r="L10" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="M10" s="12"/>
-      <c r="N10" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="O10" s="12"/>
+      <c r="I10" s="18"/>
+      <c r="J10" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="K10" s="18"/>
+      <c r="L10" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="M10" s="18"/>
+      <c r="N10" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="O10" s="18"/>
     </row>
     <row r="11" spans="2:15" ht="18" customHeight="1">
-      <c r="B11" s="6"/>
-      <c r="D11" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13" t="s">
-        <v>43</v>
-      </c>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="I11" s="13"/>
-      <c r="J11" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="K11" s="13"/>
-      <c r="L11" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="M11" s="13"/>
-      <c r="N11" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="O11" s="13"/>
+      <c r="B11" s="4"/>
+      <c r="D11" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="G11" s="19"/>
+      <c r="H11" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="I11" s="19"/>
+      <c r="J11" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="K11" s="19"/>
+      <c r="L11" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="M11" s="19"/>
+      <c r="N11" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="O11" s="19"/>
     </row>
     <row r="12" spans="2:15">
-      <c r="B12" s="6"/>
+      <c r="B12" s="4"/>
     </row>
     <row r="13" spans="2:15">
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="10" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="14" spans="2:15">
-      <c r="B14" s="6"/>
+      <c r="B14" s="4"/>
     </row>
     <row r="15" spans="2:15">
-      <c r="B15" s="6"/>
+      <c r="B15" s="4"/>
     </row>
     <row r="16" spans="2:15">
-      <c r="B16" s="6"/>
+      <c r="B16" s="10" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="17" spans="2:2">
-      <c r="B17" s="6"/>
+      <c r="B17" s="4"/>
     </row>
     <row r="18" spans="2:2">
-      <c r="B18" s="6"/>
+      <c r="B18" s="4"/>
     </row>
     <row r="19" spans="2:2">
-      <c r="B19" s="6"/>
+      <c r="B19" s="10" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="20" spans="2:2">
-      <c r="B20" s="6"/>
+      <c r="B20" s="4"/>
     </row>
     <row r="21" spans="2:2">
-      <c r="B21" s="6"/>
+      <c r="B21" s="4"/>
     </row>
     <row r="22" spans="2:2">
-      <c r="B22" s="6"/>
+      <c r="B22" s="4"/>
     </row>
     <row r="23" spans="2:2">
-      <c r="B23" s="6"/>
+      <c r="B23" s="4"/>
     </row>
     <row r="24" spans="2:2">
-      <c r="B24" s="6"/>
+      <c r="B24" s="4"/>
     </row>
     <row r="25" spans="2:2">
-      <c r="B25" s="6"/>
+      <c r="B25" s="4"/>
     </row>
     <row r="26" spans="2:2">
-      <c r="B26" s="6"/>
+      <c r="B26" s="4"/>
     </row>
     <row r="27" spans="2:2">
-      <c r="B27" s="6"/>
+      <c r="B27" s="4"/>
     </row>
     <row r="28" spans="2:2">
-      <c r="B28" s="6"/>
+      <c r="B28" s="4"/>
     </row>
     <row r="29" spans="2:2">
-      <c r="B29" s="6"/>
+      <c r="B29" s="4"/>
     </row>
     <row r="30" spans="2:2">
-      <c r="B30" s="6"/>
+      <c r="B30" s="4"/>
     </row>
     <row r="31" spans="2:2">
-      <c r="B31" s="6"/>
+      <c r="B31" s="4"/>
     </row>
     <row r="32" spans="2:2">
-      <c r="B32" s="6"/>
+      <c r="B32" s="4"/>
     </row>
     <row r="33" spans="2:2">
-      <c r="B33" s="6"/>
+      <c r="B33" s="4"/>
     </row>
     <row r="34" spans="2:2">
-      <c r="B34" s="6"/>
+      <c r="B34" s="4"/>
     </row>
     <row r="35" spans="2:2">
-      <c r="B35" s="6"/>
+      <c r="B35" s="4"/>
     </row>
     <row r="36" spans="2:2">
-      <c r="B36" s="6"/>
+      <c r="B36" s="4"/>
     </row>
     <row r="37" spans="2:2">
-      <c r="B37" s="6"/>
+      <c r="B37" s="4"/>
     </row>
     <row r="38" spans="2:2">
-      <c r="B38" s="14" t="s">
-        <v>5</v>
-      </c>
+      <c r="B38" s="4"/>
     </row>
     <row r="39" spans="2:2">
-      <c r="B39" s="4" t="s">
-        <v>6</v>
-      </c>
+      <c r="B39" s="4"/>
     </row>
     <row r="40" spans="2:2">
-      <c r="B40" s="6"/>
+      <c r="B40" s="4"/>
     </row>
     <row r="41" spans="2:2">
-      <c r="B41" s="6"/>
+      <c r="B41" s="4"/>
     </row>
     <row r="42" spans="2:2">
-      <c r="B42" s="6"/>
+      <c r="B42" s="4"/>
     </row>
     <row r="43" spans="2:2">
-      <c r="B43" s="6"/>
+      <c r="B43" s="4"/>
     </row>
     <row r="44" spans="2:2">
-      <c r="B44" s="6"/>
+      <c r="B44" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="27">
@@ -2694,17 +3148,19 @@
     <mergeCell ref="N11:O11"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B7" location="Dashboard!A1" display="📊  Dashboard"/>
-    <hyperlink ref="B10" location="Summary!A1" display="📈  Summary"/>
-    <hyperlink ref="B13" location="Data_Engine!A1" display="🗄️  Database"/>
+    <hyperlink ref="B7" location="Welcome_HQ!A1" display="🏛️  HQ Cover"/>
+    <hyperlink ref="B10" location="Dashboard!A1" display="📊  Dashboard"/>
+    <hyperlink ref="B13" location="Summary!A1" display="📈  Summary Memo"/>
+    <hyperlink ref="B16" location="Payroll_Simulator!A1" display="💰  Payroll Simulator"/>
+    <hyperlink ref="B19" location="Data_Engine!A1" display="🗄️  Data Engine"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" fitToHeight="0" orientation="landscape"/>
+  <pageSetup fitToHeight="0" orientation="landscape"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -2723,238 +3179,242 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
+      <c r="D2" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
     </row>
     <row r="3" spans="2:8">
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="2:8">
-      <c r="B4" s="6"/>
-      <c r="D4" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="16"/>
+      <c r="B4" s="4"/>
+      <c r="D4" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
     </row>
     <row r="5" spans="2:8">
-      <c r="B5" s="6"/>
-      <c r="D5" s="17" t="s">
-        <v>57</v>
-      </c>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
+      <c r="B5" s="4"/>
+      <c r="D5" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="21"/>
     </row>
     <row r="6" spans="2:8">
-      <c r="B6" s="6"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
+      <c r="B6" s="4"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="21"/>
     </row>
     <row r="7" spans="2:8">
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="10" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="8" spans="2:8">
-      <c r="B8" s="6"/>
-      <c r="D8" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="16"/>
+      <c r="B8" s="4"/>
+      <c r="D8" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
     </row>
     <row r="9" spans="2:8">
-      <c r="B9" s="6"/>
-      <c r="D9" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17"/>
+      <c r="B9" s="4"/>
+      <c r="D9" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="E9" s="21"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="21"/>
     </row>
     <row r="10" spans="2:8">
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="21"/>
+      <c r="H10" s="21"/>
     </row>
     <row r="11" spans="2:8">
-      <c r="B11" s="6"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="17"/>
+      <c r="B11" s="4"/>
+      <c r="D11" s="21"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="21"/>
+      <c r="H11" s="21"/>
     </row>
     <row r="12" spans="2:8">
-      <c r="B12" s="6"/>
+      <c r="B12" s="4"/>
     </row>
     <row r="13" spans="2:8">
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="D13" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="16"/>
-      <c r="H13" s="16"/>
+      <c r="D13" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
     </row>
     <row r="14" spans="2:8">
-      <c r="B14" s="6"/>
-      <c r="D14" s="17" t="s">
-        <v>61</v>
-      </c>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
+      <c r="B14" s="4"/>
+      <c r="D14" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="E14" s="21"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="21"/>
     </row>
     <row r="15" spans="2:8">
-      <c r="B15" s="6"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
-      <c r="G15" s="17"/>
-      <c r="H15" s="17"/>
+      <c r="B15" s="4"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="21"/>
+      <c r="H15" s="21"/>
     </row>
     <row r="16" spans="2:8">
-      <c r="B16" s="6"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="17"/>
+      <c r="B16" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D16" s="21"/>
+      <c r="E16" s="21"/>
+      <c r="F16" s="21"/>
+      <c r="G16" s="21"/>
+      <c r="H16" s="21"/>
     </row>
     <row r="17" spans="2:8">
-      <c r="B17" s="6"/>
+      <c r="B17" s="4"/>
     </row>
     <row r="18" spans="2:8">
-      <c r="B18" s="6"/>
-      <c r="D18" s="16" t="s">
-        <v>62</v>
-      </c>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="16"/>
-      <c r="H18" s="16"/>
+      <c r="B18" s="4"/>
+      <c r="D18" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="6"/>
+      <c r="H18" s="6"/>
     </row>
     <row r="19" spans="2:8">
-      <c r="B19" s="6"/>
-      <c r="D19" s="18" t="s">
-        <v>63</v>
-      </c>
-      <c r="E19" s="18"/>
-      <c r="F19" s="19" t="s">
-        <v>64</v>
-      </c>
-      <c r="G19" s="19"/>
-      <c r="H19" s="20" t="s">
-        <v>65</v>
+      <c r="B19" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="D19" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="E19" s="22"/>
+      <c r="F19" s="23" t="s">
+        <v>79</v>
+      </c>
+      <c r="G19" s="23"/>
+      <c r="H19" s="24" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="20" spans="2:8">
-      <c r="B20" s="6"/>
-      <c r="D20" s="18" t="s">
-        <v>66</v>
-      </c>
-      <c r="E20" s="18"/>
-      <c r="F20" s="19" t="s">
-        <v>67</v>
-      </c>
-      <c r="G20" s="19"/>
-      <c r="H20" s="20" t="s">
-        <v>68</v>
+      <c r="B20" s="4"/>
+      <c r="D20" s="22" t="s">
+        <v>81</v>
+      </c>
+      <c r="E20" s="22"/>
+      <c r="F20" s="23" t="s">
+        <v>82</v>
+      </c>
+      <c r="G20" s="23"/>
+      <c r="H20" s="24" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="21" spans="2:8">
-      <c r="B21" s="6"/>
-      <c r="D21" s="18" t="s">
-        <v>69</v>
-      </c>
-      <c r="E21" s="18"/>
-      <c r="F21" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="G21" s="19"/>
-      <c r="H21" s="20" t="s">
-        <v>71</v>
+      <c r="B21" s="4"/>
+      <c r="D21" s="22" t="s">
+        <v>84</v>
+      </c>
+      <c r="E21" s="22"/>
+      <c r="F21" s="23" t="s">
+        <v>85</v>
+      </c>
+      <c r="G21" s="23"/>
+      <c r="H21" s="24" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="22" spans="2:8">
-      <c r="B22" s="6"/>
-      <c r="D22" s="18" t="s">
-        <v>72</v>
-      </c>
-      <c r="E22" s="18"/>
-      <c r="F22" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="G22" s="19"/>
-      <c r="H22" s="20" t="s">
-        <v>74</v>
+      <c r="B22" s="4"/>
+      <c r="D22" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="E22" s="22"/>
+      <c r="F22" s="23" t="s">
+        <v>88</v>
+      </c>
+      <c r="G22" s="23"/>
+      <c r="H22" s="24" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="23" spans="2:8">
-      <c r="B23" s="6"/>
+      <c r="B23" s="4"/>
     </row>
     <row r="24" spans="2:8">
-      <c r="B24" s="6"/>
+      <c r="B24" s="4"/>
     </row>
     <row r="25" spans="2:8">
-      <c r="B25" s="6"/>
+      <c r="B25" s="4"/>
     </row>
     <row r="26" spans="2:8">
-      <c r="B26" s="6"/>
+      <c r="B26" s="4"/>
     </row>
     <row r="27" spans="2:8">
-      <c r="B27" s="6"/>
+      <c r="B27" s="4"/>
     </row>
     <row r="28" spans="2:8">
-      <c r="B28" s="6"/>
+      <c r="B28" s="4"/>
     </row>
     <row r="29" spans="2:8">
-      <c r="B29" s="6"/>
+      <c r="B29" s="4"/>
     </row>
     <row r="30" spans="2:8">
-      <c r="B30" s="6"/>
+      <c r="B30" s="4"/>
     </row>
     <row r="31" spans="2:8">
-      <c r="B31" s="6"/>
+      <c r="B31" s="4"/>
     </row>
     <row r="32" spans="2:8">
-      <c r="B32" s="6"/>
+      <c r="B32" s="4"/>
     </row>
     <row r="33" spans="2:2">
-      <c r="B33" s="6"/>
+      <c r="B33" s="4"/>
     </row>
     <row r="34" spans="2:2">
-      <c r="B34" s="6"/>
+      <c r="B34" s="4"/>
     </row>
     <row r="35" spans="2:2">
-      <c r="B35" s="6"/>
+      <c r="B35" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="16">
@@ -2976,16 +3436,378 @@
     <mergeCell ref="F22:G22"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B7" location="Dashboard!A1" display="📊  Dashboard"/>
-    <hyperlink ref="B10" location="Summary!A1" display="📈  Summary"/>
-    <hyperlink ref="B13" location="Data_Engine!A1" display="🗄️  Database"/>
+    <hyperlink ref="B7" location="Welcome_HQ!A1" display="🏛️  HQ Cover"/>
+    <hyperlink ref="B10" location="Dashboard!A1" display="📊  Dashboard"/>
+    <hyperlink ref="B13" location="Summary!A1" display="📈  Summary Memo"/>
+    <hyperlink ref="B16" location="Payroll_Simulator!A1" display="💰  Payroll Simulator"/>
+    <hyperlink ref="B19" location="Data_Engine!A1" display="🗄️  Data Engine"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" orientation="landscape"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B2:K30"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="2.7109375" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="3" width="2.7109375" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" customWidth="1"/>
+    <col min="5" max="5" width="18.7109375" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" customWidth="1"/>
+    <col min="8" max="10" width="14.7109375" customWidth="1"/>
+    <col min="11" max="11" width="16.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:11">
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="20"/>
+    </row>
+    <row r="3" spans="2:11">
+      <c r="B3" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:11">
+      <c r="B4" s="4"/>
+      <c r="D4" s="25" t="s">
+        <v>91</v>
+      </c>
+      <c r="E4" s="25" t="s">
+        <v>92</v>
+      </c>
+      <c r="F4" s="25" t="s">
+        <v>93</v>
+      </c>
+      <c r="G4" s="25" t="s">
+        <v>94</v>
+      </c>
+      <c r="H4" s="25" t="s">
+        <v>95</v>
+      </c>
+      <c r="I4" s="25" t="s">
+        <v>96</v>
+      </c>
+      <c r="J4" s="25" t="s">
+        <v>97</v>
+      </c>
+      <c r="K4" s="25" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11">
+      <c r="B5" s="4"/>
+      <c r="D5" s="26" t="s">
+        <v>99</v>
+      </c>
+      <c r="E5" s="26" t="s">
+        <v>100</v>
+      </c>
+      <c r="F5" s="27">
+        <v>42000</v>
+      </c>
+      <c r="G5" s="28">
+        <v>80</v>
+      </c>
+      <c r="H5" s="27">
+        <v>750</v>
+      </c>
+      <c r="I5" s="27">
+        <f>G5*H5</f>
+        <v>0</v>
+      </c>
+      <c r="J5" s="27">
+        <f>I5*0.40</f>
+        <v>0</v>
+      </c>
+      <c r="K5" s="27">
+        <f>F5+(I5*0.60)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11">
+      <c r="B6" s="4"/>
+      <c r="D6" s="26" t="s">
+        <v>101</v>
+      </c>
+      <c r="E6" s="26" t="s">
+        <v>102</v>
+      </c>
+      <c r="F6" s="27">
+        <v>38500</v>
+      </c>
+      <c r="G6" s="28">
+        <v>95</v>
+      </c>
+      <c r="H6" s="27">
+        <v>650</v>
+      </c>
+      <c r="I6" s="27">
+        <f>G6*H6</f>
+        <v>0</v>
+      </c>
+      <c r="J6" s="27">
+        <f>I6*0.40</f>
+        <v>0</v>
+      </c>
+      <c r="K6" s="27">
+        <f>F6+(I6*0.60)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11">
+      <c r="B7" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7" s="26" t="s">
+        <v>103</v>
+      </c>
+      <c r="E7" s="26" t="s">
+        <v>104</v>
+      </c>
+      <c r="F7" s="27">
+        <v>36000</v>
+      </c>
+      <c r="G7" s="28">
+        <v>70</v>
+      </c>
+      <c r="H7" s="27">
+        <v>700</v>
+      </c>
+      <c r="I7" s="27">
+        <f>G7*H7</f>
+        <v>0</v>
+      </c>
+      <c r="J7" s="27">
+        <f>I7*0.40</f>
+        <v>0</v>
+      </c>
+      <c r="K7" s="27">
+        <f>F7+(I7*0.60)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11">
+      <c r="B8" s="4"/>
+      <c r="D8" s="26" t="s">
+        <v>105</v>
+      </c>
+      <c r="E8" s="26" t="s">
+        <v>106</v>
+      </c>
+      <c r="F8" s="27">
+        <v>32000</v>
+      </c>
+      <c r="G8" s="28">
+        <v>60</v>
+      </c>
+      <c r="H8" s="27">
+        <v>600</v>
+      </c>
+      <c r="I8" s="27">
+        <f>G8*H8</f>
+        <v>0</v>
+      </c>
+      <c r="J8" s="27">
+        <f>I8*0.40</f>
+        <v>0</v>
+      </c>
+      <c r="K8" s="27">
+        <f>F8+(I8*0.60)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11">
+      <c r="B9" s="4"/>
+      <c r="D9" s="26" t="s">
+        <v>107</v>
+      </c>
+      <c r="E9" s="26" t="s">
+        <v>100</v>
+      </c>
+      <c r="F9" s="27">
+        <v>34000</v>
+      </c>
+      <c r="G9" s="28">
+        <v>85</v>
+      </c>
+      <c r="H9" s="27">
+        <v>550</v>
+      </c>
+      <c r="I9" s="27">
+        <f>G9*H9</f>
+        <v>0</v>
+      </c>
+      <c r="J9" s="27">
+        <f>I9*0.40</f>
+        <v>0</v>
+      </c>
+      <c r="K9" s="27">
+        <f>F9+(I9*0.60)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11">
+      <c r="B10" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="E10" s="26" t="s">
+        <v>109</v>
+      </c>
+      <c r="F10" s="27">
+        <v>26000</v>
+      </c>
+      <c r="G10" s="28">
+        <v>45</v>
+      </c>
+      <c r="H10" s="27">
+        <v>500</v>
+      </c>
+      <c r="I10" s="27">
+        <f>G10*H10</f>
+        <v>0</v>
+      </c>
+      <c r="J10" s="27">
+        <f>I10*0.40</f>
+        <v>0</v>
+      </c>
+      <c r="K10" s="27">
+        <f>F10+(I10*0.60)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11">
+      <c r="B11" s="4"/>
+      <c r="D11" s="25" t="s">
+        <v>110</v>
+      </c>
+      <c r="E11" s="25"/>
+      <c r="F11" s="27">
+        <f>SUM(F5:F10)</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="28">
+        <f>SUM(G5:G10)</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="I11" s="27">
+        <f>SUM(I5:I10)</f>
+        <v>0</v>
+      </c>
+      <c r="J11" s="27">
+        <f>SUM(J5:J10)</f>
+        <v>0</v>
+      </c>
+      <c r="K11" s="27">
+        <f>SUM(K5:K10)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11">
+      <c r="B12" s="4"/>
+    </row>
+    <row r="13" spans="2:11">
+      <c r="B13" s="10" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="2:11">
+      <c r="B14" s="4"/>
+    </row>
+    <row r="15" spans="2:11">
+      <c r="B15" s="4"/>
+    </row>
+    <row r="16" spans="2:11">
+      <c r="B16" s="7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2">
+      <c r="B17" s="4"/>
+    </row>
+    <row r="18" spans="2:2">
+      <c r="B18" s="4"/>
+    </row>
+    <row r="19" spans="2:2">
+      <c r="B19" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2">
+      <c r="B20" s="4"/>
+    </row>
+    <row r="21" spans="2:2">
+      <c r="B21" s="4"/>
+    </row>
+    <row r="22" spans="2:2">
+      <c r="B22" s="4"/>
+    </row>
+    <row r="23" spans="2:2">
+      <c r="B23" s="4"/>
+    </row>
+    <row r="24" spans="2:2">
+      <c r="B24" s="4"/>
+    </row>
+    <row r="25" spans="2:2">
+      <c r="B25" s="4"/>
+    </row>
+    <row r="26" spans="2:2">
+      <c r="B26" s="4"/>
+    </row>
+    <row r="27" spans="2:2">
+      <c r="B27" s="4"/>
+    </row>
+    <row r="28" spans="2:2">
+      <c r="B28" s="4"/>
+    </row>
+    <row r="29" spans="2:2">
+      <c r="B29" s="4"/>
+    </row>
+    <row r="30" spans="2:2">
+      <c r="B30" s="4"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="D2:K2"/>
+    <mergeCell ref="D11:E11"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="B7" location="Welcome_HQ!A1" display="🏛️  HQ Cover"/>
+    <hyperlink ref="B10" location="Dashboard!A1" display="📊  Dashboard"/>
+    <hyperlink ref="B13" location="Summary!A1" display="📈  Summary Memo"/>
+    <hyperlink ref="B16" location="Payroll_Simulator!A1" display="💰  Payroll Simulator"/>
+    <hyperlink ref="B19" location="Data_Engine!A1" display="🗄️  Data Engine"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup fitToHeight="0" orientation="landscape"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2994,298 +3816,298 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="21" t="s">
-        <v>75</v>
-      </c>
-      <c r="B1" s="21" t="s">
+      <c r="A1" s="25" t="s">
+        <v>112</v>
+      </c>
+      <c r="B1" s="25" t="s">
+        <v>113</v>
+      </c>
+      <c r="C1" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="E1" s="25" t="s">
+        <v>118</v>
+      </c>
+      <c r="F1" s="25" t="s">
+        <v>119</v>
+      </c>
+      <c r="G1" s="25" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="28">
+        <v>28</v>
+      </c>
+      <c r="C2" s="29">
+        <v>0.062</v>
+      </c>
+      <c r="E2" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="F2" s="28">
+        <v>42</v>
+      </c>
+      <c r="G2" s="28">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="26" t="s">
+        <v>115</v>
+      </c>
+      <c r="B3" s="28">
+        <v>47</v>
+      </c>
+      <c r="C3" s="29">
+        <v>0.104</v>
+      </c>
+      <c r="E3" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="F3" s="28">
+        <v>90</v>
+      </c>
+      <c r="G3" s="28">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="26" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" s="28">
+        <v>58</v>
+      </c>
+      <c r="C4" s="29">
+        <v>0.128</v>
+      </c>
+      <c r="E4" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="F4" s="28">
+        <v>161</v>
+      </c>
+      <c r="G4" s="28">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="26" t="s">
+        <v>116</v>
+      </c>
+      <c r="B5" s="28">
+        <v>83</v>
+      </c>
+      <c r="C5" s="29">
+        <v>0.183</v>
+      </c>
+      <c r="E5" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="F5" s="28">
+        <v>247</v>
+      </c>
+      <c r="G5" s="28">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="28">
+        <v>104</v>
+      </c>
+      <c r="C6" s="29">
+        <v>0.229</v>
+      </c>
+      <c r="E6" s="26" t="s">
+        <v>51</v>
+      </c>
+      <c r="F6" s="28">
+        <v>284</v>
+      </c>
+      <c r="G6" s="28">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="26" t="s">
+        <v>117</v>
+      </c>
+      <c r="B7" s="28">
+        <v>134</v>
+      </c>
+      <c r="C7" s="29">
+        <v>0.295</v>
+      </c>
+      <c r="E7" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="F7" s="28">
+        <v>321</v>
+      </c>
+      <c r="G7" s="28">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="25" t="s">
+        <v>112</v>
+      </c>
+      <c r="B10" s="25" t="s">
+        <v>121</v>
+      </c>
+      <c r="E10" s="25" t="s">
+        <v>127</v>
+      </c>
+      <c r="F10" s="25" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="26" t="s">
+        <v>122</v>
+      </c>
+      <c r="B11" s="29">
+        <v>0.39</v>
+      </c>
+      <c r="E11" s="26" t="s">
+        <v>129</v>
+      </c>
+      <c r="F11" s="28">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="26" t="s">
+        <v>123</v>
+      </c>
+      <c r="B12" s="29">
+        <v>0.3</v>
+      </c>
+      <c r="E12" s="26" t="s">
+        <v>130</v>
+      </c>
+      <c r="F12" s="28">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="26" t="s">
+        <v>124</v>
+      </c>
+      <c r="B13" s="29">
+        <v>0.29</v>
+      </c>
+      <c r="E13" s="26" t="s">
+        <v>131</v>
+      </c>
+      <c r="F13" s="28">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" s="26" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" s="29">
+        <v>0.25</v>
+      </c>
+      <c r="E14" s="26" t="s">
+        <v>132</v>
+      </c>
+      <c r="F14" s="28">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" s="26" t="s">
+        <v>125</v>
+      </c>
+      <c r="B15" s="29">
+        <v>0.12</v>
+      </c>
+      <c r="E15" s="26" t="s">
+        <v>133</v>
+      </c>
+      <c r="F15" s="28">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" s="26" t="s">
+        <v>126</v>
+      </c>
+      <c r="B16" s="29">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="25" t="s">
+        <v>134</v>
+      </c>
+      <c r="B18" s="25" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19" s="28">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="B20" s="28">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="26" t="s">
+        <v>37</v>
+      </c>
+      <c r="B21" s="28">
         <v>76</v>
       </c>
-      <c r="C1" s="21" t="s">
-        <v>77</v>
-      </c>
-      <c r="E1" s="21" t="s">
-        <v>81</v>
-      </c>
-      <c r="F1" s="21" t="s">
-        <v>82</v>
-      </c>
-      <c r="G1" s="21" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" s="23">
-        <v>28</v>
-      </c>
-      <c r="C2" s="24">
-        <v>0.062</v>
-      </c>
-      <c r="E2" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="F2" s="23">
-        <v>42</v>
-      </c>
-      <c r="G2" s="23">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="22" t="s">
-        <v>78</v>
-      </c>
-      <c r="B3" s="23">
-        <v>47</v>
-      </c>
-      <c r="C3" s="24">
-        <v>0.104</v>
-      </c>
-      <c r="E3" s="22" t="s">
-        <v>33</v>
-      </c>
-      <c r="F3" s="23">
-        <v>90</v>
-      </c>
-      <c r="G3" s="23">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" s="23">
-        <v>58</v>
-      </c>
-      <c r="C4" s="24">
-        <v>0.128</v>
-      </c>
-      <c r="E4" s="22" t="s">
-        <v>34</v>
-      </c>
-      <c r="F4" s="23">
-        <v>161</v>
-      </c>
-      <c r="G4" s="23">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="22" t="s">
-        <v>79</v>
-      </c>
-      <c r="B5" s="23">
-        <v>83</v>
-      </c>
-      <c r="C5" s="24">
-        <v>0.183</v>
-      </c>
-      <c r="E5" s="22" t="s">
-        <v>35</v>
-      </c>
-      <c r="F5" s="23">
-        <v>247</v>
-      </c>
-      <c r="G5" s="23">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="22" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="23">
-        <v>104</v>
-      </c>
-      <c r="C6" s="24">
-        <v>0.229</v>
-      </c>
-      <c r="E6" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="F6" s="23">
-        <v>284</v>
-      </c>
-      <c r="G6" s="23">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="22" t="s">
-        <v>80</v>
-      </c>
-      <c r="B7" s="23">
-        <v>134</v>
-      </c>
-      <c r="C7" s="24">
-        <v>0.295</v>
-      </c>
-      <c r="E7" s="22" t="s">
-        <v>37</v>
-      </c>
-      <c r="F7" s="23">
-        <v>321</v>
-      </c>
-      <c r="G7" s="23">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="A10" s="21" t="s">
-        <v>75</v>
-      </c>
-      <c r="B10" s="21" t="s">
-        <v>84</v>
-      </c>
-      <c r="E10" s="21" t="s">
-        <v>90</v>
-      </c>
-      <c r="F10" s="21" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="A11" s="22" t="s">
-        <v>85</v>
-      </c>
-      <c r="B11" s="24">
-        <v>0.39</v>
-      </c>
-      <c r="E11" s="22" t="s">
-        <v>92</v>
-      </c>
-      <c r="F11" s="23">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="A12" s="22" t="s">
-        <v>86</v>
-      </c>
-      <c r="B12" s="24">
-        <v>0.3</v>
-      </c>
-      <c r="E12" s="22" t="s">
-        <v>93</v>
-      </c>
-      <c r="F12" s="23">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="A13" s="22" t="s">
-        <v>87</v>
-      </c>
-      <c r="B13" s="24">
-        <v>0.29</v>
-      </c>
-      <c r="E13" s="22" t="s">
-        <v>94</v>
-      </c>
-      <c r="F13" s="23">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
-      <c r="A14" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" s="24">
-        <v>0.25</v>
-      </c>
-      <c r="E14" s="22" t="s">
-        <v>95</v>
-      </c>
-      <c r="F14" s="23">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
-      <c r="A15" s="22" t="s">
-        <v>88</v>
-      </c>
-      <c r="B15" s="24">
-        <v>0.12</v>
-      </c>
-      <c r="E15" s="22" t="s">
-        <v>96</v>
-      </c>
-      <c r="F15" s="23">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
-      <c r="A16" s="22" t="s">
-        <v>89</v>
-      </c>
-      <c r="B16" s="24">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2">
-      <c r="A18" s="21" t="s">
-        <v>97</v>
-      </c>
-      <c r="B18" s="21" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2">
-      <c r="A19" s="22" t="s">
-        <v>17</v>
-      </c>
-      <c r="B19" s="23">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2">
-      <c r="A20" s="22" t="s">
-        <v>18</v>
-      </c>
-      <c r="B20" s="23">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2">
-      <c r="A21" s="22" t="s">
-        <v>19</v>
-      </c>
-      <c r="B21" s="23">
-        <v>76</v>
-      </c>
     </row>
     <row r="22" spans="1:2">
-      <c r="A22" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="B22" s="23">
+      <c r="A22" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="B22" s="28">
         <v>68</v>
       </c>
     </row>
     <row r="23" spans="1:2">
-      <c r="A23" s="22" t="s">
-        <v>99</v>
-      </c>
-      <c r="B23" s="23">
+      <c r="A23" s="26" t="s">
+        <v>136</v>
+      </c>
+      <c r="B23" s="28">
         <v>54</v>
       </c>
     </row>
     <row r="24" spans="1:2">
-      <c r="A24" s="22" t="s">
-        <v>100</v>
-      </c>
-      <c r="B24" s="23">
+      <c r="A24" s="26" t="s">
+        <v>137</v>
+      </c>
+      <c r="B24" s="28">
         <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:2">
-      <c r="A25" s="22" t="s">
-        <v>101</v>
-      </c>
-      <c r="B25" s="23">
+      <c r="A25" s="26" t="s">
+        <v>138</v>
+      </c>
+      <c r="B25" s="28">
         <v>32</v>
       </c>
     </row>

</xml_diff>